<commit_message>
feedback page and link updates
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{43B5458B-67A6-401E-8364-7A5B684416D4}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0F506B-5F19-4ED5-A820-352740C36564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-38520" yWindow="-5340" windowWidth="38640" windowHeight="21120" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-37500" yWindow="-3855" windowWidth="23010" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -33,7 +33,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="530">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1160" uniqueCount="529">
   <si>
     <t>interview</t>
   </si>
@@ -2713,9 +2713,6 @@
     <t>Rate</t>
   </si>
   <si>
-    <t>Calificar</t>
-  </si>
-  <si>
     <t>cde408e1c1e11192688bbf2538317637</t>
   </si>
   <si>
@@ -3121,9 +3118,6 @@
 </t>
   </si>
   <si>
-    <t>Retroalimentación enviada</t>
-  </si>
-  <si>
     <t>6fed7ad2098d5420c544911762581296</t>
   </si>
   <si>
@@ -3553,39 +3547,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>¿Preguntas o comentarios? [**Contacte a ILAO**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>https://es.illinoislegalaid.org/contact-us</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>).</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Si tienes más que decir, [**contacta a ILAO**](</t>
     </r>
     <r>
       <rPr>
@@ -10028,212 +9989,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>${ action_button_html(url_action('review_answers'), label=word(':edit: Edit answers'), color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>% endif
-% endif
-% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if not user_logged_in():
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Iniciar sesión**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('login', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>) o [**crear**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('register', next=interview_url())}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">) una cuenta de ILAO Easy Form para **guardar tu progreso**.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-¿Comentarios, sugerencias u observaciones? [**Cuéntanos :external-link:**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ interview_url(i='docassemble.ILAO:feedback.yml',easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">){:target='_blank'}.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if nav.get_section() != None:
-% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
-% if current_context().question_id == None:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% elif "review screen" not in current_context().question_id:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
     </r>
     <r>
       <rPr>
@@ -10593,37 +10348,265 @@
 ${ collapse_template(al_formatted_error_message) }</t>
   </si>
   <si>
-    <t>¿Qué Formulario Fácil utilizaste?</t>
-  </si>
-  <si>
-    <t>Retroalimentación de Formulario Fácil</t>
-  </si>
-  <si>
     <t>Revisa el número de teléfono e inténtalo de nuevo. Si el número es de fuera de los Estados Unidos, empieza con un signo "+" y luego ingresa el código de país y el número de teléfono.</t>
   </si>
   <si>
+    <t>Comentarios sobre el Formulario Fácil</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Si tienes más comentarios,  [**comunícate con ILAO**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>https://es.illinoislegalaid.org/contact-us</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>).</t>
+    </r>
+  </si>
+  <si>
     <t>% if easy_form_session_info_not_found == True:
-Cuéntanos qué te parece el Formulario Fácil
+Dinos qué piensas del Formulario Fácil.
 % else:
-Cuéntanos qué te parece el **${ url_args.get('easy_form_title') }** Formulario Fácil.
+Dinos qué piensas del Formulario Fácil de **${ url_args.get('easy_form_title') }**.
 % endif</t>
   </si>
   <si>
-    <t>% if easy_form_session_info_not_found == True:
-**La información de Formulario Fácil no se cargó automáticamente.**
-Título de Formulario Fácil (seleccionado por el usuario): ${ easy_form_selection }
-Página de lanzamiento de ILAO Formulario Fácil: ${ easy_forms_info(easy_form_selection)['url'] }
-% else:
-Título de Formulario Fácil: ${ url_args.get('easy_form_title') }
-Página de lanzamiento de ILAO Formulario Fácil: ${ url_args.get('easy_form_interview') }
+    <t>¿Qué Formulario Fácil usaste?</t>
+  </si>
+  <si>
+    <t>Califica</t>
+  </si>
+  <si>
+    <t>Comentarios enviados</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if not user_logged_in():
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>[${fa_icon('sign-in-alt', color='#0079d0', size='sm')} **Iniciar sesión**]</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>(</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('login', next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>) o [**crear**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('register', lang="es", next=interview_url())}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">) una cuenta de ILAO Easy Form para **guardar tu progreso**.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+¿Comentarios, sugerencias u observaciones? [**Cuéntanos :external-link:**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ interview_url(i='docassemble.ILAO:feedback.yml', lang="es", easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">){:target='_blank'}.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if nav.get_section() != None:
+% if nav.get_section() != 'section_intro' and nav.get_section() != 'section_download':
+% if current_context().question_id == None:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% elif "review screen" not in current_context().question_id:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ action_button_html(url_action('review_answers'), label=':edit: Editar respuestas', color='success', size='md') }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>% endif
 % endif
-Correo electrónico del usuario: ${ user.email }
-Comentarios del usuario: ${ feedback }
-Calificación: ${ rating }
---- Información de depuración ---
-Página de la entrevista: ${ url_args.get('easy_form_page') }
-Variable buscada (si la hay): ${ url_args.get('easy_form_variable') }
-Mensaje de error: ${ urllib.parse.unquote(url_args.get('easy_form_error_message', '')) }</t>
+% endif</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -11083,7 +11066,7 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B2" s="5" t="s">
         <v>288</v>
@@ -11101,15 +11084,15 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>379</v>
+        <v>376</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>522</v>
+        <v>518</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B3" s="5" t="s">
         <v>288</v>
@@ -11127,15 +11110,15 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B4" s="5" t="s">
         <v>288</v>
@@ -11144,7 +11127,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>496</v>
+        <v>492</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11153,15 +11136,15 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>494</v>
+        <v>491</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>495</v>
+        <v>528</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B5" s="5" t="s">
         <v>288</v>
@@ -11170,7 +11153,7 @@
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
-        <v>362</v>
+        <v>359</v>
       </c>
       <c r="E5" s="5" t="s">
         <v>8</v>
@@ -11179,24 +11162,24 @@
         <v>9</v>
       </c>
       <c r="G5" s="6" t="s">
-        <v>363</v>
+        <v>360</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>469</v>
+        <v>466</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
-        <v>486</v>
+        <v>483</v>
       </c>
       <c r="E6" s="5" t="s">
         <v>8</v>
@@ -11205,24 +11188,24 @@
         <v>9</v>
       </c>
       <c r="G6" s="6" t="s">
-        <v>487</v>
+        <v>484</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>488</v>
+        <v>485</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>497</v>
+        <v>493</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>8</v>
@@ -11231,24 +11214,24 @@
         <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>508</v>
+        <v>504</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>498</v>
+        <v>494</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>8</v>
@@ -11257,24 +11240,24 @@
         <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>509</v>
+        <v>505</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>512</v>
+        <v>508</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>8</v>
@@ -11283,24 +11266,24 @@
         <v>9</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>515</v>
+        <v>511</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>510</v>
+        <v>506</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>513</v>
+        <v>509</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>8</v>
@@ -11309,24 +11292,24 @@
         <v>9</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>516</v>
+        <v>512</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>511</v>
+        <v>507</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>514</v>
+        <v>510</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>8</v>
@@ -11335,7 +11318,7 @@
         <v>9</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>517</v>
+        <v>513</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>297</v>
@@ -11343,16 +11326,16 @@
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
       </c>
       <c r="D12" s="5" t="s">
-        <v>502</v>
+        <v>498</v>
       </c>
       <c r="E12" s="5" t="s">
         <v>8</v>
@@ -11361,24 +11344,24 @@
         <v>9</v>
       </c>
       <c r="G12" s="6" t="s">
-        <v>503</v>
+        <v>499</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>504</v>
+        <v>500</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>366</v>
+        <v>363</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>485</v>
+        <v>482</v>
       </c>
       <c r="C13" s="5">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="s">
-        <v>505</v>
+        <v>501</v>
       </c>
       <c r="E13" s="5" t="s">
         <v>8</v>
@@ -11387,15 +11370,15 @@
         <v>9</v>
       </c>
       <c r="G13" s="6" t="s">
-        <v>506</v>
+        <v>502</v>
       </c>
       <c r="H13" s="2" t="s">
-        <v>507</v>
+        <v>503</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
@@ -11421,7 +11404,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -11439,15 +11422,15 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>364</v>
+        <v>361</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>358</v>
+        <v>355</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -11473,7 +11456,7 @@
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -11494,12 +11477,12 @@
         <v>54</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>352</v>
+        <v>349</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -11517,7 +11500,7 @@
         <v>9</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>365</v>
+        <v>362</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>223</v>
@@ -11525,7 +11508,7 @@
     </row>
     <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
@@ -11546,12 +11529,12 @@
         <v>58</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>468</v>
+        <v>465</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -11577,7 +11560,7 @@
     </row>
     <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -11595,15 +11578,15 @@
         <v>9</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>353</v>
+        <v>350</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>467</v>
+        <v>464</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -11629,7 +11612,7 @@
     </row>
     <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
@@ -11647,15 +11630,15 @@
         <v>9</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>354</v>
+        <v>351</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>466</v>
+        <v>463</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
@@ -11681,7 +11664,7 @@
     </row>
     <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
@@ -11699,15 +11682,15 @@
         <v>9</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>355</v>
+        <v>352</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>464</v>
+        <v>461</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
@@ -11733,7 +11716,7 @@
     </row>
     <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -11751,15 +11734,15 @@
         <v>9</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>356</v>
+        <v>353</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>463</v>
+        <v>460</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
@@ -11785,7 +11768,7 @@
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
@@ -11811,7 +11794,7 @@
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -11837,7 +11820,7 @@
     </row>
     <row r="31" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -11858,12 +11841,12 @@
         <v>42</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>462</v>
+        <v>459</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -11884,12 +11867,12 @@
         <v>44</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>465</v>
+        <v>462</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -11915,7 +11898,7 @@
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
@@ -11941,7 +11924,7 @@
     </row>
     <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
@@ -11967,7 +11950,7 @@
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
@@ -11993,7 +11976,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -12014,12 +11997,12 @@
         <v>54</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>357</v>
+        <v>354</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -12045,7 +12028,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -12071,7 +12054,7 @@
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -12092,12 +12075,12 @@
         <v>60</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>461</v>
+        <v>458</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -12123,7 +12106,7 @@
     </row>
     <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
@@ -12149,7 +12132,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
@@ -12175,7 +12158,7 @@
     </row>
     <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
@@ -12201,7 +12184,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
@@ -12227,7 +12210,7 @@
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
@@ -12253,7 +12236,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
@@ -12279,7 +12262,7 @@
     </row>
     <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
@@ -12305,7 +12288,7 @@
     </row>
     <row r="49" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
@@ -12331,7 +12314,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
@@ -12357,7 +12340,7 @@
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
@@ -12378,12 +12361,12 @@
         <v>82</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>460</v>
+        <v>457</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
@@ -12409,7 +12392,7 @@
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -12435,7 +12418,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -12461,7 +12444,7 @@
     </row>
     <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -12482,12 +12465,12 @@
         <v>90</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>458</v>
+        <v>455</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -12513,7 +12496,7 @@
     </row>
     <row r="57" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>14</v>
@@ -12534,12 +12517,12 @@
         <v>94</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>459</v>
+        <v>456</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>14</v>
@@ -12565,7 +12548,7 @@
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>14</v>
@@ -12591,7 +12574,7 @@
     </row>
     <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>14</v>
@@ -12617,7 +12600,7 @@
     </row>
     <row r="61" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>14</v>
@@ -12643,7 +12626,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>14</v>
@@ -12669,7 +12652,7 @@
     </row>
     <row r="63" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>14</v>
@@ -12695,7 +12678,7 @@
     </row>
     <row r="64" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>107</v>
@@ -12721,7 +12704,7 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>107</v>
@@ -12730,7 +12713,7 @@
         <v>1</v>
       </c>
       <c r="D65" s="5" t="s">
-        <v>482</v>
+        <v>479</v>
       </c>
       <c r="E65" s="5" t="s">
         <v>8</v>
@@ -12739,15 +12722,15 @@
         <v>9</v>
       </c>
       <c r="G65" s="6" t="s">
-        <v>483</v>
+        <v>480</v>
       </c>
       <c r="H65" s="2" t="s">
-        <v>484</v>
+        <v>481</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>110</v>
@@ -12773,7 +12756,7 @@
     </row>
     <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>113</v>
@@ -12799,7 +12782,7 @@
     </row>
     <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>113</v>
@@ -12825,7 +12808,7 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>113</v>
@@ -12851,7 +12834,7 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>113</v>
@@ -12877,7 +12860,7 @@
     </row>
     <row r="71" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>113</v>
@@ -12903,7 +12886,7 @@
     </row>
     <row r="72" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>113</v>
@@ -12929,16 +12912,16 @@
     </row>
     <row r="73" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>501</v>
+        <v>497</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>499</v>
+        <v>495</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>8</v>
@@ -12947,15 +12930,15 @@
         <v>9</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>500</v>
+        <v>496</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>527</v>
+        <v>521</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>12</v>
@@ -12981,7 +12964,7 @@
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>12</v>
@@ -13007,7 +12990,7 @@
     </row>
     <row r="76" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>12</v>
@@ -13033,7 +13016,7 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>12</v>
@@ -13059,7 +13042,7 @@
     </row>
     <row r="78" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>12</v>
@@ -13085,7 +13068,7 @@
     </row>
     <row r="79" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>12</v>
@@ -13111,7 +13094,7 @@
     </row>
     <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>138</v>
@@ -13137,7 +13120,7 @@
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>138</v>
@@ -13163,7 +13146,7 @@
     </row>
     <row r="82" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>143</v>
@@ -13184,12 +13167,12 @@
         <v>145</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>523</v>
+        <v>519</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>143</v>
@@ -13215,7 +13198,7 @@
     </row>
     <row r="84" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>10</v>
@@ -13236,12 +13219,12 @@
         <v>149</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>433</v>
+        <v>430</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>150</v>
@@ -13267,7 +13250,7 @@
     </row>
     <row r="86" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>150</v>
@@ -13293,7 +13276,7 @@
     </row>
     <row r="87" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>155</v>
@@ -13319,7 +13302,7 @@
     </row>
     <row r="88" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>155</v>
@@ -13340,12 +13323,12 @@
         <v>159</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>453</v>
+        <v>450</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>160</v>
@@ -13371,7 +13354,7 @@
     </row>
     <row r="90" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>160</v>
@@ -13397,7 +13380,7 @@
     </row>
     <row r="91" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>160</v>
@@ -13418,12 +13401,12 @@
         <v>166</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>480</v>
+        <v>477</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>160</v>
@@ -13449,7 +13432,7 @@
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>160</v>
@@ -13470,12 +13453,12 @@
         <v>170</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>470</v>
+        <v>467</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>171</v>
@@ -13496,12 +13479,12 @@
         <v>173</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>476</v>
+        <v>473</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>171</v>
@@ -13522,12 +13505,12 @@
         <v>175</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>454</v>
+        <v>451</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>11</v>
@@ -13545,15 +13528,15 @@
         <v>9</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>368</v>
+        <v>365</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>481</v>
+        <v>478</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
-        <v>489</v>
+        <v>486</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>10</v>
@@ -13562,7 +13545,7 @@
         <v>1</v>
       </c>
       <c r="D97" s="5" t="s">
-        <v>490</v>
+        <v>487</v>
       </c>
       <c r="E97" s="5" t="s">
         <v>8</v>
@@ -13571,15 +13554,15 @@
         <v>9</v>
       </c>
       <c r="G97" s="6" t="s">
-        <v>492</v>
+        <v>489</v>
       </c>
       <c r="H97" s="2" t="s">
-        <v>491</v>
+        <v>488</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>11</v>
@@ -13605,7 +13588,7 @@
     </row>
     <row r="99" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>179</v>
@@ -13631,7 +13614,7 @@
     </row>
     <row r="100" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>179</v>
@@ -13652,12 +13635,12 @@
         <v>183</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>455</v>
+        <v>452</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>184</v>
@@ -13683,7 +13666,7 @@
     </row>
     <row r="102" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>184</v>
@@ -13709,7 +13692,7 @@
     </row>
     <row r="103" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>184</v>
@@ -13735,7 +13718,7 @@
     </row>
     <row r="104" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>184</v>
@@ -13761,7 +13744,7 @@
     </row>
     <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>184</v>
@@ -13787,7 +13770,7 @@
     </row>
     <row r="106" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>184</v>
@@ -13813,7 +13796,7 @@
     </row>
     <row r="107" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>197</v>
@@ -13839,7 +13822,7 @@
     </row>
     <row r="108" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>197</v>
@@ -13865,7 +13848,7 @@
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>202</v>
@@ -13883,15 +13866,15 @@
         <v>9</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>473</v>
+        <v>470</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>472</v>
+        <v>469</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>202</v>
@@ -13909,15 +13892,15 @@
         <v>9</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>351</v>
+        <v>348</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>493</v>
+        <v>490</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>205</v>
@@ -13935,15 +13918,15 @@
         <v>9</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>471</v>
+        <v>468</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>477</v>
+        <v>474</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>207</v>
@@ -13961,7 +13944,7 @@
         <v>9</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>478</v>
+        <v>475</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>260</v>
@@ -13969,7 +13952,7 @@
     </row>
     <row r="113" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
-        <v>367</v>
+        <v>364</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>209</v>
@@ -13987,7 +13970,7 @@
         <v>9</v>
       </c>
       <c r="G113" s="6" t="s">
-        <v>479</v>
+        <v>476</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>261</v>
@@ -13995,7 +13978,7 @@
     </row>
     <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>211</v>
@@ -14013,15 +13996,15 @@
         <v>9</v>
       </c>
       <c r="G114" s="6" t="s">
-        <v>359</v>
+        <v>356</v>
       </c>
       <c r="H114" s="3" t="s">
-        <v>360</v>
+        <v>357</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>211</v>
@@ -14042,12 +14025,12 @@
         <v>214</v>
       </c>
       <c r="H115" s="3" t="s">
-        <v>361</v>
+        <v>358</v>
       </c>
     </row>
     <row r="116" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>215</v>
@@ -14068,12 +14051,12 @@
         <v>217</v>
       </c>
       <c r="H116" s="2" t="s">
-        <v>349</v>
+        <v>347</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>218</v>
@@ -14094,12 +14077,12 @@
         <v>220</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>348</v>
+        <v>346</v>
       </c>
     </row>
     <row r="118" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>218</v>
@@ -14108,7 +14091,7 @@
         <v>1</v>
       </c>
       <c r="D118" s="5" t="s">
-        <v>518</v>
+        <v>514</v>
       </c>
       <c r="E118" s="5" t="s">
         <v>8</v>
@@ -14117,15 +14100,15 @@
         <v>9</v>
       </c>
       <c r="G118" s="6" t="s">
-        <v>519</v>
+        <v>515</v>
       </c>
       <c r="H118" s="3" t="s">
-        <v>520</v>
-      </c>
-    </row>
-    <row r="119" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="119" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B119" s="5" t="s">
         <v>291</v>
@@ -14134,7 +14117,7 @@
         <v>0</v>
       </c>
       <c r="D119" s="5" t="s">
-        <v>373</v>
+        <v>370</v>
       </c>
       <c r="E119" s="5" t="s">
         <v>8</v>
@@ -14143,15 +14126,15 @@
         <v>9</v>
       </c>
       <c r="G119" s="6" t="s">
-        <v>374</v>
+        <v>371</v>
       </c>
       <c r="H119" s="2" t="s">
-        <v>522</v>
-      </c>
-    </row>
-    <row r="120" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
+        <v>518</v>
+      </c>
+    </row>
+    <row r="120" spans="1:8" ht="225" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B120" s="5" t="s">
         <v>291</v>
@@ -14160,7 +14143,7 @@
         <v>1</v>
       </c>
       <c r="D120" s="5" t="s">
-        <v>375</v>
+        <v>372</v>
       </c>
       <c r="E120" s="5" t="s">
         <v>8</v>
@@ -14169,15 +14152,15 @@
         <v>9</v>
       </c>
       <c r="G120" s="6" t="s">
-        <v>376</v>
+        <v>373</v>
       </c>
       <c r="H120" s="2" t="s">
-        <v>521</v>
+        <v>517</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A121" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B121" s="5" t="s">
         <v>291</v>
@@ -14198,12 +14181,12 @@
         <v>293</v>
       </c>
       <c r="H121" s="2" t="s">
-        <v>350</v>
+        <v>523</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B122" s="5" t="s">
         <v>294</v>
@@ -14229,7 +14212,7 @@
     </row>
     <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B123" s="5" t="s">
         <v>294</v>
@@ -14250,12 +14233,12 @@
         <v>299</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>526</v>
+        <v>522</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B124" s="5" t="s">
         <v>294</v>
@@ -14276,12 +14259,12 @@
         <v>301</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>528</v>
+        <v>524</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B125" s="5" t="s">
         <v>294</v>
@@ -14307,7 +14290,7 @@
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B126" s="5" t="s">
         <v>294</v>
@@ -14333,7 +14316,7 @@
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B127" s="5" t="s">
         <v>294</v>
@@ -14354,12 +14337,12 @@
         <v>308</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>309</v>
+        <v>526</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B128" s="5" t="s">
         <v>294</v>
@@ -14368,24 +14351,24 @@
         <v>6</v>
       </c>
       <c r="D128" s="5" t="s">
+        <v>309</v>
+      </c>
+      <c r="E128" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F128" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G128" s="6" t="s">
         <v>310</v>
       </c>
-      <c r="E128" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F128" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G128" s="6" t="s">
+      <c r="H128" s="2" t="s">
         <v>311</v>
-      </c>
-      <c r="H128" s="2" t="s">
-        <v>312</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B129" s="5" t="s">
         <v>294</v>
@@ -14394,76 +14377,76 @@
         <v>7</v>
       </c>
       <c r="D129" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F129" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G129" s="6" t="s">
         <v>313</v>
       </c>
-      <c r="E129" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G129" s="6" t="s">
+      <c r="H129" s="2" t="s">
         <v>314</v>
-      </c>
-      <c r="H129" s="2" t="s">
-        <v>315</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>316</v>
+        <v>315</v>
       </c>
       <c r="C130" s="5">
         <v>0</v>
       </c>
       <c r="D130" s="5" t="s">
+        <v>316</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G130" s="6" t="s">
         <v>317</v>
       </c>
-      <c r="E130" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F130" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G130" s="6" t="s">
-        <v>318</v>
-      </c>
-      <c r="H130" s="2" t="s">
-        <v>529</v>
+      <c r="H130" s="6" t="s">
+        <v>317</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="C131" s="5">
         <v>0</v>
       </c>
       <c r="D131" s="5" t="s">
+        <v>319</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G131" s="6" t="s">
         <v>320</v>
       </c>
-      <c r="E131" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F131" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G131" s="6" t="s">
-        <v>321</v>
-      </c>
       <c r="H131" s="3" t="s">
-        <v>322</v>
+        <v>527</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B132" s="5" t="s">
         <v>11</v>
@@ -14472,24 +14455,24 @@
         <v>0</v>
       </c>
       <c r="D132" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F132" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G132" s="6" t="s">
+        <v>322</v>
+      </c>
+      <c r="H132" s="2" t="s">
         <v>323</v>
-      </c>
-      <c r="E132" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F132" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G132" s="6" t="s">
-        <v>324</v>
-      </c>
-      <c r="H132" s="2" t="s">
-        <v>325</v>
       </c>
     </row>
     <row r="133" spans="1:8" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>11</v>
@@ -14498,7 +14481,7 @@
         <v>1</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>474</v>
+        <v>471</v>
       </c>
       <c r="E133" s="5" t="s">
         <v>8</v>
@@ -14507,15 +14490,15 @@
         <v>9</v>
       </c>
       <c r="G133" s="6" t="s">
-        <v>475</v>
+        <v>472</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>524</v>
+        <v>520</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>11</v>
@@ -14524,24 +14507,24 @@
         <v>2</v>
       </c>
       <c r="D134" s="5" t="s">
+        <v>324</v>
+      </c>
+      <c r="E134" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G134" s="6" t="s">
+        <v>325</v>
+      </c>
+      <c r="H134" s="2" t="s">
         <v>326</v>
-      </c>
-      <c r="E134" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F134" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G134" s="6" t="s">
-        <v>327</v>
-      </c>
-      <c r="H134" s="2" t="s">
-        <v>328</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="5" t="s">
-        <v>370</v>
+        <v>367</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>11</v>
@@ -14567,16 +14550,16 @@
     </row>
     <row r="136" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A136" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C136" s="5">
         <v>0</v>
       </c>
       <c r="D136" s="5" t="s">
-        <v>383</v>
+        <v>380</v>
       </c>
       <c r="E136" s="5" t="s">
         <v>8</v>
@@ -14585,24 +14568,24 @@
         <v>9</v>
       </c>
       <c r="G136" s="6" t="s">
-        <v>384</v>
+        <v>381</v>
       </c>
       <c r="H136" s="8" t="s">
-        <v>445</v>
+        <v>442</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A137" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C137" s="5">
         <v>1</v>
       </c>
       <c r="D137" s="5" t="s">
-        <v>385</v>
+        <v>382</v>
       </c>
       <c r="E137" s="5" t="s">
         <v>8</v>
@@ -14611,24 +14594,24 @@
         <v>9</v>
       </c>
       <c r="G137" s="6" t="s">
-        <v>386</v>
+        <v>383</v>
       </c>
       <c r="H137" s="2" t="s">
-        <v>442</v>
+        <v>439</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>382</v>
+        <v>379</v>
       </c>
       <c r="C138" s="5">
         <v>2</v>
       </c>
       <c r="D138" s="5" t="s">
-        <v>387</v>
+        <v>384</v>
       </c>
       <c r="E138" s="5" t="s">
         <v>8</v>
@@ -14637,24 +14620,24 @@
         <v>9</v>
       </c>
       <c r="G138" s="6" t="s">
-        <v>388</v>
+        <v>385</v>
       </c>
       <c r="H138" s="2" t="s">
-        <v>444</v>
+        <v>441</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C139" s="5">
         <v>0</v>
       </c>
       <c r="D139" s="5" t="s">
-        <v>389</v>
+        <v>386</v>
       </c>
       <c r="E139" s="5" t="s">
         <v>8</v>
@@ -14663,22 +14646,22 @@
         <v>9</v>
       </c>
       <c r="G139" s="6" t="s">
-        <v>390</v>
+        <v>387</v>
       </c>
       <c r="H139" s="7"/>
     </row>
     <row r="140" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C140" s="5">
         <v>1</v>
       </c>
       <c r="D140" s="5" t="s">
-        <v>391</v>
+        <v>388</v>
       </c>
       <c r="E140" s="5" t="s">
         <v>8</v>
@@ -14687,24 +14670,24 @@
         <v>9</v>
       </c>
       <c r="G140" s="6" t="s">
-        <v>392</v>
+        <v>389</v>
       </c>
       <c r="H140" s="2" t="s">
-        <v>440</v>
+        <v>437</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C141" s="5">
         <v>2</v>
       </c>
       <c r="D141" s="5" t="s">
-        <v>393</v>
+        <v>390</v>
       </c>
       <c r="E141" s="5" t="s">
         <v>8</v>
@@ -14713,24 +14696,24 @@
         <v>9</v>
       </c>
       <c r="G141" s="6" t="s">
-        <v>394</v>
+        <v>391</v>
       </c>
       <c r="H141" s="2" t="s">
-        <v>456</v>
+        <v>453</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C142" s="5">
         <v>3</v>
       </c>
       <c r="D142" s="5" t="s">
-        <v>395</v>
+        <v>392</v>
       </c>
       <c r="E142" s="5" t="s">
         <v>8</v>
@@ -14739,15 +14722,15 @@
         <v>9</v>
       </c>
       <c r="G142" s="6" t="s">
-        <v>396</v>
+        <v>393</v>
       </c>
       <c r="H142" s="2" t="s">
-        <v>457</v>
+        <v>454</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B143" s="5" t="s">
         <v>171</v>
@@ -14756,7 +14739,7 @@
         <v>0</v>
       </c>
       <c r="D143" s="5" t="s">
-        <v>397</v>
+        <v>394</v>
       </c>
       <c r="E143" s="5" t="s">
         <v>8</v>
@@ -14765,13 +14748,13 @@
         <v>9</v>
       </c>
       <c r="G143" s="6" t="s">
-        <v>398</v>
+        <v>395</v>
       </c>
       <c r="H143" s="7"/>
     </row>
     <row r="144" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A144" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B144" s="5" t="s">
         <v>171</v>
@@ -14780,7 +14763,7 @@
         <v>1</v>
       </c>
       <c r="D144" s="5" t="s">
-        <v>399</v>
+        <v>396</v>
       </c>
       <c r="E144" s="5" t="s">
         <v>8</v>
@@ -14789,15 +14772,15 @@
         <v>9</v>
       </c>
       <c r="G144" s="6" t="s">
-        <v>400</v>
+        <v>397</v>
       </c>
       <c r="H144" s="2" t="s">
-        <v>441</v>
+        <v>438</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A145" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B145" s="5" t="s">
         <v>171</v>
@@ -14806,7 +14789,7 @@
         <v>2</v>
       </c>
       <c r="D145" s="5" t="s">
-        <v>401</v>
+        <v>398</v>
       </c>
       <c r="E145" s="5" t="s">
         <v>8</v>
@@ -14815,15 +14798,15 @@
         <v>9</v>
       </c>
       <c r="G145" s="6" t="s">
-        <v>402</v>
+        <v>399</v>
       </c>
       <c r="H145" s="2" t="s">
-        <v>432</v>
+        <v>429</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B146" s="5" t="s">
         <v>171</v>
@@ -14832,7 +14815,7 @@
         <v>3</v>
       </c>
       <c r="D146" s="5" t="s">
-        <v>403</v>
+        <v>400</v>
       </c>
       <c r="E146" s="5" t="s">
         <v>8</v>
@@ -14841,15 +14824,15 @@
         <v>9</v>
       </c>
       <c r="G146" s="6" t="s">
-        <v>404</v>
+        <v>401</v>
       </c>
       <c r="H146" s="2" t="s">
-        <v>430</v>
+        <v>427</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>171</v>
@@ -14858,7 +14841,7 @@
         <v>4</v>
       </c>
       <c r="D147" s="5" t="s">
-        <v>405</v>
+        <v>402</v>
       </c>
       <c r="E147" s="5" t="s">
         <v>8</v>
@@ -14867,24 +14850,24 @@
         <v>9</v>
       </c>
       <c r="G147" s="6" t="s">
-        <v>406</v>
+        <v>403</v>
       </c>
       <c r="H147" s="2" t="s">
-        <v>431</v>
+        <v>428</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C148" s="5">
         <v>0</v>
       </c>
       <c r="D148" s="5" t="s">
-        <v>408</v>
+        <v>405</v>
       </c>
       <c r="E148" s="5" t="s">
         <v>8</v>
@@ -14893,22 +14876,22 @@
         <v>9</v>
       </c>
       <c r="G148" s="6" t="s">
-        <v>409</v>
+        <v>406</v>
       </c>
       <c r="H148" s="7"/>
     </row>
     <row r="149" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A149" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C149" s="5">
         <v>1</v>
       </c>
       <c r="D149" s="5" t="s">
-        <v>410</v>
+        <v>407</v>
       </c>
       <c r="E149" s="5" t="s">
         <v>8</v>
@@ -14917,24 +14900,24 @@
         <v>9</v>
       </c>
       <c r="G149" s="6" t="s">
-        <v>411</v>
+        <v>408</v>
       </c>
       <c r="H149" s="2" t="s">
-        <v>443</v>
+        <v>440</v>
       </c>
     </row>
     <row r="150" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A150" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>407</v>
+        <v>404</v>
       </c>
       <c r="C150" s="5">
         <v>2</v>
       </c>
       <c r="D150" s="5" t="s">
-        <v>412</v>
+        <v>409</v>
       </c>
       <c r="E150" s="5" t="s">
         <v>8</v>
@@ -14943,24 +14926,24 @@
         <v>9</v>
       </c>
       <c r="G150" s="6" t="s">
-        <v>413</v>
+        <v>410</v>
       </c>
       <c r="H150" s="2" t="s">
-        <v>446</v>
+        <v>443</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A151" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="C151" s="5">
         <v>0</v>
       </c>
       <c r="D151" s="5" t="s">
-        <v>415</v>
+        <v>412</v>
       </c>
       <c r="E151" s="5" t="s">
         <v>8</v>
@@ -14969,24 +14952,24 @@
         <v>9</v>
       </c>
       <c r="G151" s="6" t="s">
-        <v>416</v>
+        <v>413</v>
       </c>
       <c r="H151" s="2" t="s">
-        <v>439</v>
+        <v>436</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A152" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="C152" s="5">
         <v>1</v>
       </c>
       <c r="D152" s="5" t="s">
-        <v>417</v>
+        <v>414</v>
       </c>
       <c r="E152" s="5" t="s">
         <v>8</v>
@@ -14995,24 +14978,24 @@
         <v>9</v>
       </c>
       <c r="G152" s="6" t="s">
-        <v>418</v>
+        <v>415</v>
       </c>
       <c r="H152" s="2" t="s">
-        <v>438</v>
+        <v>435</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A153" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>414</v>
+        <v>411</v>
       </c>
       <c r="C153" s="5">
         <v>2</v>
       </c>
       <c r="D153" s="5" t="s">
-        <v>419</v>
+        <v>416</v>
       </c>
       <c r="E153" s="5" t="s">
         <v>8</v>
@@ -15021,24 +15004,24 @@
         <v>9</v>
       </c>
       <c r="G153" s="6" t="s">
-        <v>420</v>
+        <v>417</v>
       </c>
       <c r="H153" s="2" t="s">
-        <v>437</v>
+        <v>434</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A154" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C154" s="5">
         <v>0</v>
       </c>
       <c r="D154" s="5" t="s">
-        <v>421</v>
+        <v>418</v>
       </c>
       <c r="E154" s="5" t="s">
         <v>8</v>
@@ -15047,24 +15030,24 @@
         <v>9</v>
       </c>
       <c r="G154" s="6" t="s">
-        <v>422</v>
+        <v>419</v>
       </c>
       <c r="H154" s="2" t="s">
-        <v>436</v>
+        <v>433</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A155" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C155" s="5">
         <v>1</v>
       </c>
       <c r="D155" s="5" t="s">
-        <v>423</v>
+        <v>420</v>
       </c>
       <c r="E155" s="5" t="s">
         <v>8</v>
@@ -15073,24 +15056,24 @@
         <v>9</v>
       </c>
       <c r="G155" s="6" t="s">
-        <v>424</v>
+        <v>421</v>
       </c>
       <c r="H155" s="2" t="s">
-        <v>435</v>
+        <v>432</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C156" s="5">
         <v>2</v>
       </c>
       <c r="D156" s="5" t="s">
-        <v>425</v>
+        <v>422</v>
       </c>
       <c r="E156" s="5" t="s">
         <v>8</v>
@@ -15099,24 +15082,24 @@
         <v>9</v>
       </c>
       <c r="G156" s="6" t="s">
-        <v>426</v>
+        <v>423</v>
       </c>
       <c r="H156" s="2" t="s">
-        <v>434</v>
+        <v>431</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A157" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>427</v>
+        <v>424</v>
       </c>
       <c r="C157" s="5">
         <v>0</v>
       </c>
       <c r="D157" s="5" t="s">
-        <v>428</v>
+        <v>425</v>
       </c>
       <c r="E157" s="5" t="s">
         <v>8</v>
@@ -15125,24 +15108,24 @@
         <v>9</v>
       </c>
       <c r="G157" s="6" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
       <c r="H157" s="2" t="s">
-        <v>429</v>
+        <v>426</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A158" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C158" s="5">
         <v>0</v>
       </c>
       <c r="D158" s="5" t="s">
-        <v>380</v>
+        <v>377</v>
       </c>
       <c r="E158" s="5" t="s">
         <v>8</v>
@@ -15151,24 +15134,24 @@
         <v>9</v>
       </c>
       <c r="G158" s="6" t="s">
-        <v>381</v>
+        <v>378</v>
       </c>
       <c r="H158" s="3" t="s">
-        <v>330</v>
+        <v>328</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A159" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>329</v>
+        <v>327</v>
       </c>
       <c r="C159" s="5">
         <v>1</v>
       </c>
       <c r="D159" s="5" t="s">
-        <v>331</v>
+        <v>329</v>
       </c>
       <c r="E159" s="5" t="s">
         <v>8</v>
@@ -15177,24 +15160,24 @@
         <v>9</v>
       </c>
       <c r="G159" s="6" t="s">
-        <v>332</v>
+        <v>330</v>
       </c>
       <c r="H159" s="2" t="s">
-        <v>377</v>
+        <v>374</v>
       </c>
     </row>
     <row r="160" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A160" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C160" s="5">
         <v>0</v>
       </c>
       <c r="D160" s="5" t="s">
-        <v>334</v>
+        <v>332</v>
       </c>
       <c r="E160" s="5" t="s">
         <v>8</v>
@@ -15203,24 +15186,24 @@
         <v>9</v>
       </c>
       <c r="G160" s="6" t="s">
-        <v>335</v>
+        <v>333</v>
       </c>
       <c r="H160" s="2" t="s">
-        <v>372</v>
+        <v>369</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A161" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C161" s="5">
         <v>1</v>
       </c>
       <c r="D161" s="5" t="s">
-        <v>336</v>
+        <v>334</v>
       </c>
       <c r="E161" s="5" t="s">
         <v>8</v>
@@ -15229,24 +15212,24 @@
         <v>9</v>
       </c>
       <c r="G161" s="6" t="s">
-        <v>378</v>
+        <v>375</v>
       </c>
       <c r="H161" s="2" t="s">
-        <v>449</v>
+        <v>446</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A162" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>333</v>
+        <v>331</v>
       </c>
       <c r="C162" s="5">
         <v>2</v>
       </c>
       <c r="D162" s="5" t="s">
-        <v>337</v>
+        <v>335</v>
       </c>
       <c r="E162" s="5" t="s">
         <v>8</v>
@@ -15255,93 +15238,93 @@
         <v>9</v>
       </c>
       <c r="G162" s="6" t="s">
-        <v>447</v>
+        <v>444</v>
       </c>
       <c r="H162" s="2" t="s">
-        <v>448</v>
+        <v>445</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A163" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C163" s="5">
         <v>0</v>
       </c>
       <c r="D163" s="5" t="s">
+        <v>337</v>
+      </c>
+      <c r="E163" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F163" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G163" s="6" t="s">
+        <v>338</v>
+      </c>
+      <c r="H163" s="2" t="s">
         <v>339</v>
-      </c>
-      <c r="E163" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F163" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G163" s="6" t="s">
-        <v>340</v>
-      </c>
-      <c r="H163" s="2" t="s">
-        <v>341</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A164" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C164" s="5">
         <v>1</v>
       </c>
       <c r="D164" s="5" t="s">
+        <v>340</v>
+      </c>
+      <c r="E164" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F164" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G164" s="6" t="s">
+        <v>341</v>
+      </c>
+      <c r="H164" s="3" t="s">
         <v>342</v>
-      </c>
-      <c r="E164" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F164" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G164" s="6" t="s">
-        <v>343</v>
-      </c>
-      <c r="H164" s="3" t="s">
-        <v>344</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A165" s="5" t="s">
-        <v>371</v>
+        <v>368</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>338</v>
+        <v>336</v>
       </c>
       <c r="C165" s="5">
         <v>2</v>
       </c>
       <c r="D165" s="5" t="s">
+        <v>343</v>
+      </c>
+      <c r="E165" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F165" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G165" s="6" t="s">
+        <v>344</v>
+      </c>
+      <c r="H165" s="3" t="s">
         <v>345</v>
-      </c>
-      <c r="E165" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F165" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G165" s="6" t="s">
-        <v>346</v>
-      </c>
-      <c r="H165" s="3" t="s">
-        <v>347</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A166" s="5" t="s">
-        <v>369</v>
+        <v>366</v>
       </c>
       <c r="B166" s="5" t="s">
         <v>215</v>
@@ -15350,7 +15333,7 @@
         <v>1</v>
       </c>
       <c r="D166" s="5" t="s">
-        <v>450</v>
+        <v>447</v>
       </c>
       <c r="E166" s="5" t="s">
         <v>8</v>
@@ -15359,10 +15342,10 @@
         <v>9</v>
       </c>
       <c r="G166" s="6" t="s">
-        <v>451</v>
+        <v>448</v>
       </c>
       <c r="H166" s="2" t="s">
-        <v>452</v>
+        <v>449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
url arg adjustments for Spanish version > Feedback
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{4E0F506B-5F19-4ED5-A820-352740C36564}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BC5ACB-45BD-4EE3-9179-52CCB4EA1FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37500" yWindow="-3855" windowWidth="23010" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -9744,14 +9744,6 @@
     <t>Para continuar, debes aceptar los [**términos de uso**](https://es.illinoislegalaid.org/about/terms-of-use) y la [**política de privacidad**](https://es.illinoislegalaid.org/about/privacy-policy).</t>
   </si>
   <si>
-    <t>Se produjo un error al intentar cargar esta pantalla.
-Puedes probar alguno de estos pasos para recuperar tu trabajo:
-* Haz clic en **Atrás** y vuelve a intentarlo,
-* [:comment-dots: **Cuéntanos qué pasó**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url , easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=action_argument('error_message'), local=False,reset=1) }){target="_blank"}, o
-* Visita la [**ILAO Form Library**](https://es.illinoislegalaid.org/form-library) y prueba otro Easy Form.
-${ collapse_template(al_formatted_error_message) }</t>
-  </si>
-  <si>
     <t>56e6ddd1cb6cec596b433440dfb21c17</t>
   </si>
   <si>
@@ -10340,14 +10332,6 @@
     <t>Tienes respuestas guardadas disponibles para este Formulario Fácil.</t>
   </si>
   <si>
-    <t>Se produjo un error al intentar cargar esta pantalla.
-Puedes intentar uno de estos pasos para recuperar tu trabajo:
-* Haz clic en **Atrás** y vuelve a intentarlo,
-* [:comment-dots: **Cuéntenos qué pasó.**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url , easy_form_title=ilao_easy_form_title, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }){target="_blank"}, o
-* Visita la [**Biblioteca de formularios de ILAO**](https://es.illinoislegalaid.org/form-library) y prueba otro Formulario Fácil.
-${ collapse_template(al_formatted_error_message) }</t>
-  </si>
-  <si>
     <t>Revisa el número de teléfono e inténtalo de nuevo. Si el número es de fuera de los Estados Unidos, empieza con un signo "+" y luego ingresa el código de país y el número de teléfono.</t>
   </si>
   <si>
@@ -10511,7 +10495,7 @@
         <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>${ interview_url(i='docassemble.ILAO:feedback.yml', lang="es", easy_form_interview=ilao_easy_form_url,easy_form_title=ilao_easy_form_title,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
+      <t>${ interview_url(i='docassemble.ILAO:feedback.yml', lang="es", easy_form_interview=ilao_easy_form_url_es,easy_form_title=ilao_easy_form_title_es,easy_form_page=current_context().question_id,easy_form_variable=current_context().variable,local=False,reset=1) }</t>
     </r>
     <r>
       <rPr>
@@ -10607,6 +10591,22 @@
 % endif
 % endif</t>
     </r>
+  </si>
+  <si>
+    <t>Se produjo un error al intentar cargar esta pantalla.
+Puedes probar alguno de estos pasos para recuperar tu trabajo:
+* Haz clic en **Atrás** y vuelve a intentarlo,
+* [:comment-dots: **Cuéntanos qué pasó**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url_es , easy_form_title=ilao_easy_form_title_es, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=action_argument('error_message'), local=False,reset=1) }){target="_blank"}, o
+* Visita la [**ILAO Form Library**](https://es.illinoislegalaid.org/form-library) y prueba otro Easy Form.
+${ collapse_template(al_formatted_error_message) }</t>
+  </si>
+  <si>
+    <t>Se produjo un error al intentar cargar esta pantalla.
+Puedes intentar uno de estos pasos para recuperar tu trabajo:
+* Haz clic en **Atrás** y vuelve a intentarlo,
+* [:comment-dots: **Cuéntenos qué pasó.**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url_es , easy_form_title=ilao_easy_form_title_es, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }){target="_blank"}, o
+* Visita la [**Biblioteca de formularios de ILAO**](https://es.illinoislegalaid.org/form-library) y prueba otro Formulario Fácil.
+${ collapse_template(al_formatted_error_message) }</t>
   </si>
 </sst>
 </file>
@@ -11087,7 +11087,7 @@
         <v>376</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
@@ -11113,7 +11113,7 @@
         <v>373</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
@@ -11127,7 +11127,7 @@
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>492</v>
+        <v>491</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11136,10 +11136,10 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>491</v>
+        <v>490</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
@@ -11173,25 +11173,25 @@
         <v>363</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>482</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="6" t="s">
         <v>483</v>
       </c>
-      <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="6" t="s">
+      <c r="H6" s="2" t="s">
         <v>484</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>485</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
@@ -11199,13 +11199,13 @@
         <v>363</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>493</v>
+        <v>492</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>8</v>
@@ -11214,10 +11214,10 @@
         <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
-        <v>504</v>
+        <v>503</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
@@ -11225,13 +11225,13 @@
         <v>363</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>494</v>
+        <v>493</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>8</v>
@@ -11240,10 +11240,10 @@
         <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
-        <v>505</v>
+        <v>504</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -11251,13 +11251,13 @@
         <v>363</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>508</v>
+        <v>507</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>8</v>
@@ -11266,10 +11266,10 @@
         <v>9</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>511</v>
+        <v>510</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>506</v>
+        <v>505</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -11277,13 +11277,13 @@
         <v>363</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>509</v>
+        <v>508</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>8</v>
@@ -11292,10 +11292,10 @@
         <v>9</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>512</v>
+        <v>511</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>507</v>
+        <v>506</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -11303,13 +11303,13 @@
         <v>363</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>510</v>
+        <v>509</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>8</v>
@@ -11318,7 +11318,7 @@
         <v>9</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>513</v>
+        <v>512</v>
       </c>
       <c r="H11" s="2" t="s">
         <v>297</v>
@@ -11329,25 +11329,25 @@
         <v>363</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>497</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="6" t="s">
         <v>498</v>
       </c>
-      <c r="E12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="6" t="s">
+      <c r="H12" s="2" t="s">
         <v>499</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>500</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -11355,25 +11355,25 @@
         <v>363</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>482</v>
+        <v>481</v>
       </c>
       <c r="C13" s="5">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>500</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" s="6" t="s">
         <v>501</v>
       </c>
-      <c r="E13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G13" s="6" t="s">
+      <c r="H13" s="2" t="s">
         <v>502</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>503</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -12713,19 +12713,19 @@
         <v>1</v>
       </c>
       <c r="D65" s="5" t="s">
+        <v>478</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G65" s="6" t="s">
         <v>479</v>
       </c>
-      <c r="E65" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G65" s="6" t="s">
+      <c r="H65" s="2" t="s">
         <v>480</v>
-      </c>
-      <c r="H65" s="2" t="s">
-        <v>481</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -12915,25 +12915,25 @@
         <v>364</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>497</v>
+        <v>496</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
       </c>
       <c r="D73" s="5" t="s">
+        <v>494</v>
+      </c>
+      <c r="E73" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F73" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G73" s="9" t="s">
         <v>495</v>
       </c>
-      <c r="E73" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F73" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G73" s="9" t="s">
-        <v>496</v>
-      </c>
       <c r="H73" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
@@ -13167,7 +13167,7 @@
         <v>145</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>519</v>
+        <v>518</v>
       </c>
     </row>
     <row r="83" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -13508,7 +13508,7 @@
         <v>451</v>
       </c>
     </row>
-    <row r="96" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:8" ht="304.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
         <v>364</v>
       </c>
@@ -13531,12 +13531,12 @@
         <v>365</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>478</v>
+        <v>527</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
-        <v>486</v>
+        <v>485</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>10</v>
@@ -13545,19 +13545,19 @@
         <v>1</v>
       </c>
       <c r="D97" s="5" t="s">
+        <v>486</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G97" s="6" t="s">
+        <v>488</v>
+      </c>
+      <c r="H97" s="2" t="s">
         <v>487</v>
-      </c>
-      <c r="E97" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F97" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G97" s="6" t="s">
-        <v>489</v>
-      </c>
-      <c r="H97" s="2" t="s">
-        <v>488</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
@@ -13895,7 +13895,7 @@
         <v>348</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>490</v>
+        <v>489</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -14091,19 +14091,19 @@
         <v>1</v>
       </c>
       <c r="D118" s="5" t="s">
+        <v>513</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F118" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G118" s="6" t="s">
         <v>514</v>
       </c>
-      <c r="E118" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F118" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G118" s="6" t="s">
+      <c r="H118" s="3" t="s">
         <v>515</v>
-      </c>
-      <c r="H118" s="3" t="s">
-        <v>516</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.3">
@@ -14129,7 +14129,7 @@
         <v>371</v>
       </c>
       <c r="H119" s="2" t="s">
-        <v>518</v>
+        <v>517</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="225" customHeight="1" x14ac:dyDescent="0.3">
@@ -14155,7 +14155,7 @@
         <v>373</v>
       </c>
       <c r="H120" s="2" t="s">
-        <v>517</v>
+        <v>516</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
@@ -14181,7 +14181,7 @@
         <v>293</v>
       </c>
       <c r="H121" s="2" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
@@ -14233,7 +14233,7 @@
         <v>299</v>
       </c>
       <c r="H123" s="3" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.3">
@@ -14259,7 +14259,7 @@
         <v>301</v>
       </c>
       <c r="H124" s="2" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
@@ -14285,7 +14285,7 @@
         <v>303</v>
       </c>
       <c r="H125" s="3" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
@@ -14337,7 +14337,7 @@
         <v>308</v>
       </c>
       <c r="H127" s="3" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.3">
@@ -14441,7 +14441,7 @@
         <v>320</v>
       </c>
       <c r="H131" s="3" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
@@ -14493,7 +14493,7 @@
         <v>472</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>520</v>
+        <v>528</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">

</xml_diff>

<commit_message>
interview list saved easy form text translations
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{06BC5ACB-45BD-4EE3-9179-52CCB4EA1FEE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623215B1-0F92-4197-9BCF-ECBEC70D26C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-37500" yWindow="-3855" windowWidth="23010" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -1847,158 +1847,6 @@
   <si>
     <r>
       <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% for interview in interview_list(filename=current_interview_url)[0]:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${'!@&lt;a class="xyz" href="' + interview_url(i=current_interview_url, session=interview['session']) + '"&gt;!@' +  interview['title'] +  (' (' + interview.get("subtitle",'') + ')' if interview.get('subtitle') else '')  +"!@&lt;/a&gt;!@" }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  Last visited </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${format_date(interview['modtime'])}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, currently on page **</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${interview['dict'].get('_internal',{}).get('steps')}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endfor
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>[**View all of your saved Easy Forms**]</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>(</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('interviews')}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
         <sz val="11"/>
         <color rgb="FF000000"/>
         <rFont val="Calibri"/>
@@ -8125,410 +7973,6 @@
         <scheme val="minor"/>
       </rPr>
       <t>% endif</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
-% if get_config("interview page pre"):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ get_config("interview page pre") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Haz clic en el nombre de un Formulario Fácil para seguir trabajando en él o para descargar tus formularios completados.
-Usa la acción de etiqueta </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:tag:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> para agregar o editar una descripción.
-**Nota: Los Formularios Fácil se eliminan después de 90 días de inactividad.** Si quieres conservarlos por más tiempo, descarga tus formularios o reanuda el Formulario Fácil para restablecer el temporizador de actividad. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;nav aria-label="Page navigation"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if session_page &gt; 0:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Previo</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Próximo</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/ul&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/nav&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">You do not have any Easy Forms in progress.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
     </r>
   </si>
   <si>
@@ -10607,6 +10051,542 @@
 * [:comment-dots: **Cuéntenos qué pasó.**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url_es , easy_form_title=ilao_easy_form_title_es, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }){target="_blank"}, o
 * Visita la [**Biblioteca de formularios de ILAO**](https://es.illinoislegalaid.org/form-library) y prueba otro Formulario Fácil.
 ${ collapse_template(al_formatted_error_message) }</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
+% if get_config("interview page pre"):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ get_config("interview page pre") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Haz clic en el nombre de un Formulario Fácil para seguir trabajando en él o para descargar tus formularios completados.
+Usa la acción de etiqueta </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:tag:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para agregar o editar una descripción.
+**Nota: Los Formularios Fácil se eliminan después de 90 días de inactividad.** Si quieres conservarlos por más tiempo, descarga tus formularios o reanuda el Formulario Fácil para restablecer el temporizador de actividad. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;nav aria-label="Page navigation"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if session_page &gt; 0:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Previo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Próximo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/ul&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/nav&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">No tienes ningún Formulario Fácil a medias.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% for interview in interview_list(filename=current_interview_url)[0]:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${'!@&lt;a class="xyz" href="' + interview_url(i=current_interview_url, session=interview['session']) + '"&gt;!@' +  interview['title'] +  (' (' + interview.get("subtitle",'') + ')' if interview.get('subtitle') else '')  +"!@&lt;/a&gt;!@" }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  Última visita </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${format_date(interview['modtime'])}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, actualmente en la página **</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${interview['dict'].get('_internal',{}).get('steps')}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endfor
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+[**Ver todos tus Formularios Fáciles guardados**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('interviews')}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -11066,16 +11046,16 @@
     </row>
     <row r="2" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A2" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B2" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C2" s="5">
         <v>0</v>
       </c>
       <c r="D2" s="5" t="s">
-        <v>289</v>
+        <v>288</v>
       </c>
       <c r="E2" s="5" t="s">
         <v>8</v>
@@ -11084,24 +11064,24 @@
         <v>9</v>
       </c>
       <c r="G2" s="6" t="s">
-        <v>376</v>
+        <v>375</v>
       </c>
       <c r="H2" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="3" spans="1:8" ht="135" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A3" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B3" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C3" s="5">
         <v>1</v>
       </c>
       <c r="D3" s="5" t="s">
-        <v>290</v>
+        <v>289</v>
       </c>
       <c r="E3" s="5" t="s">
         <v>8</v>
@@ -11110,24 +11090,24 @@
         <v>9</v>
       </c>
       <c r="G3" s="6" t="s">
-        <v>373</v>
+        <v>372</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="4" spans="1:8" ht="345.6" x14ac:dyDescent="0.3">
       <c r="A4" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B4" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C4" s="5">
         <v>5</v>
       </c>
       <c r="D4" s="5" t="s">
-        <v>491</v>
+        <v>489</v>
       </c>
       <c r="E4" s="5" t="s">
         <v>8</v>
@@ -11136,76 +11116,76 @@
         <v>9</v>
       </c>
       <c r="G4" s="6" t="s">
-        <v>490</v>
+        <v>488</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>526</v>
+        <v>524</v>
       </c>
     </row>
     <row r="5" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A5" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B5" s="5" t="s">
-        <v>288</v>
+        <v>287</v>
       </c>
       <c r="C5" s="5">
         <v>6</v>
       </c>
       <c r="D5" s="5" t="s">
+        <v>358</v>
+      </c>
+      <c r="E5" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F5" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G5" s="6" t="s">
         <v>359</v>
       </c>
-      <c r="E5" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F5" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="6" t="s">
-        <v>360</v>
-      </c>
       <c r="H5" s="2" t="s">
-        <v>466</v>
+        <v>464</v>
       </c>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A6" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B6" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C6" s="5">
         <v>6</v>
       </c>
       <c r="D6" s="5" t="s">
+        <v>480</v>
+      </c>
+      <c r="E6" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F6" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G6" s="6" t="s">
+        <v>481</v>
+      </c>
+      <c r="H6" s="2" t="s">
         <v>482</v>
-      </c>
-      <c r="E6" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="6" t="s">
-        <v>483</v>
-      </c>
-      <c r="H6" s="2" t="s">
-        <v>484</v>
       </c>
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A7" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B7" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C7" s="5">
         <v>0</v>
       </c>
       <c r="D7" s="5" t="s">
-        <v>492</v>
+        <v>490</v>
       </c>
       <c r="E7" s="5" t="s">
         <v>8</v>
@@ -11214,24 +11194,24 @@
         <v>9</v>
       </c>
       <c r="G7" s="6" t="s">
+        <v>501</v>
+      </c>
+      <c r="H7" s="2" t="s">
         <v>503</v>
-      </c>
-      <c r="H7" s="2" t="s">
-        <v>505</v>
       </c>
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A8" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B8" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C8" s="5">
         <v>0</v>
       </c>
       <c r="D8" s="5" t="s">
-        <v>493</v>
+        <v>491</v>
       </c>
       <c r="E8" s="5" t="s">
         <v>8</v>
@@ -11240,24 +11220,24 @@
         <v>9</v>
       </c>
       <c r="G8" s="6" t="s">
+        <v>502</v>
+      </c>
+      <c r="H8" s="2" t="s">
         <v>504</v>
-      </c>
-      <c r="H8" s="2" t="s">
-        <v>506</v>
       </c>
     </row>
     <row r="9" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A9" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B9" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C9" s="5">
         <v>0</v>
       </c>
       <c r="D9" s="5" t="s">
-        <v>507</v>
+        <v>505</v>
       </c>
       <c r="E9" s="5" t="s">
         <v>8</v>
@@ -11266,24 +11246,24 @@
         <v>9</v>
       </c>
       <c r="G9" s="6" t="s">
-        <v>510</v>
+        <v>508</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>505</v>
+        <v>503</v>
       </c>
     </row>
     <row r="10" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A10" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B10" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C10" s="5">
         <v>0</v>
       </c>
       <c r="D10" s="5" t="s">
-        <v>508</v>
+        <v>506</v>
       </c>
       <c r="E10" s="5" t="s">
         <v>8</v>
@@ -11292,24 +11272,24 @@
         <v>9</v>
       </c>
       <c r="G10" s="6" t="s">
-        <v>511</v>
+        <v>509</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>506</v>
+        <v>504</v>
       </c>
     </row>
     <row r="11" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A11" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B11" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C11" s="5">
         <v>0</v>
       </c>
       <c r="D11" s="5" t="s">
-        <v>509</v>
+        <v>507</v>
       </c>
       <c r="E11" s="5" t="s">
         <v>8</v>
@@ -11318,67 +11298,67 @@
         <v>9</v>
       </c>
       <c r="G11" s="6" t="s">
-        <v>512</v>
+        <v>510</v>
       </c>
       <c r="H11" s="2" t="s">
-        <v>297</v>
+        <v>296</v>
       </c>
     </row>
     <row r="12" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A12" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C12" s="5">
         <v>0</v>
       </c>
       <c r="D12" s="5" t="s">
+        <v>495</v>
+      </c>
+      <c r="E12" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F12" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G12" s="6" t="s">
+        <v>496</v>
+      </c>
+      <c r="H12" s="2" t="s">
         <v>497</v>
-      </c>
-      <c r="E12" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F12" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="6" t="s">
-        <v>498</v>
-      </c>
-      <c r="H12" s="2" t="s">
-        <v>499</v>
       </c>
     </row>
     <row r="13" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A13" s="5" t="s">
-        <v>363</v>
+        <v>362</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>481</v>
+        <v>479</v>
       </c>
       <c r="C13" s="5">
         <v>0</v>
       </c>
       <c r="D13" s="5" t="s">
+        <v>498</v>
+      </c>
+      <c r="E13" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F13" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G13" s="6" t="s">
+        <v>499</v>
+      </c>
+      <c r="H13" s="2" t="s">
         <v>500</v>
-      </c>
-      <c r="E13" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F13" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G13" s="6" t="s">
-        <v>501</v>
-      </c>
-      <c r="H13" s="2" t="s">
-        <v>502</v>
       </c>
     </row>
     <row r="14" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A14" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B14" s="5" t="s">
         <v>14</v>
@@ -11404,7 +11384,7 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A15" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B15" s="5" t="s">
         <v>14</v>
@@ -11422,15 +11402,15 @@
         <v>9</v>
       </c>
       <c r="G15" s="6" t="s">
-        <v>361</v>
+        <v>360</v>
       </c>
       <c r="H15" s="3" t="s">
-        <v>355</v>
+        <v>354</v>
       </c>
     </row>
     <row r="16" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A16" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B16" s="5" t="s">
         <v>14</v>
@@ -11456,7 +11436,7 @@
     </row>
     <row r="17" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A17" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B17" s="5" t="s">
         <v>14</v>
@@ -11477,12 +11457,12 @@
         <v>54</v>
       </c>
       <c r="H17" s="3" t="s">
-        <v>349</v>
+        <v>348</v>
       </c>
     </row>
     <row r="18" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A18" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B18" s="5" t="s">
         <v>14</v>
@@ -11500,7 +11480,7 @@
         <v>9</v>
       </c>
       <c r="G18" s="6" t="s">
-        <v>362</v>
+        <v>361</v>
       </c>
       <c r="H18" s="3" t="s">
         <v>223</v>
@@ -11508,7 +11488,7 @@
     </row>
     <row r="19" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A19" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B19" s="5" t="s">
         <v>14</v>
@@ -11529,12 +11509,12 @@
         <v>58</v>
       </c>
       <c r="H19" s="3" t="s">
-        <v>465</v>
+        <v>463</v>
       </c>
     </row>
     <row r="20" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A20" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B20" s="5" t="s">
         <v>14</v>
@@ -11560,7 +11540,7 @@
     </row>
     <row r="21" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A21" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B21" s="5" t="s">
         <v>14</v>
@@ -11578,15 +11558,15 @@
         <v>9</v>
       </c>
       <c r="G21" s="6" t="s">
-        <v>350</v>
+        <v>349</v>
       </c>
       <c r="H21" s="3" t="s">
-        <v>464</v>
+        <v>462</v>
       </c>
     </row>
     <row r="22" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A22" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B22" s="5" t="s">
         <v>14</v>
@@ -11612,7 +11592,7 @@
     </row>
     <row r="23" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A23" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B23" s="5" t="s">
         <v>14</v>
@@ -11630,15 +11610,15 @@
         <v>9</v>
       </c>
       <c r="G23" s="6" t="s">
-        <v>351</v>
+        <v>350</v>
       </c>
       <c r="H23" s="3" t="s">
-        <v>463</v>
+        <v>461</v>
       </c>
     </row>
     <row r="24" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A24" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B24" s="5" t="s">
         <v>14</v>
@@ -11664,7 +11644,7 @@
     </row>
     <row r="25" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A25" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B25" s="5" t="s">
         <v>14</v>
@@ -11682,15 +11662,15 @@
         <v>9</v>
       </c>
       <c r="G25" s="6" t="s">
-        <v>352</v>
+        <v>351</v>
       </c>
       <c r="H25" s="3" t="s">
-        <v>461</v>
+        <v>459</v>
       </c>
     </row>
     <row r="26" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A26" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B26" s="5" t="s">
         <v>14</v>
@@ -11716,7 +11696,7 @@
     </row>
     <row r="27" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A27" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B27" s="5" t="s">
         <v>14</v>
@@ -11734,15 +11714,15 @@
         <v>9</v>
       </c>
       <c r="G27" s="6" t="s">
-        <v>353</v>
+        <v>352</v>
       </c>
       <c r="H27" s="3" t="s">
-        <v>460</v>
+        <v>458</v>
       </c>
     </row>
     <row r="28" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A28" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B28" s="5" t="s">
         <v>14</v>
@@ -11768,7 +11748,7 @@
     </row>
     <row r="29" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A29" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B29" s="5" t="s">
         <v>14</v>
@@ -11794,7 +11774,7 @@
     </row>
     <row r="30" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A30" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B30" s="5" t="s">
         <v>14</v>
@@ -11820,7 +11800,7 @@
     </row>
     <row r="31" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A31" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B31" s="5" t="s">
         <v>14</v>
@@ -11841,12 +11821,12 @@
         <v>42</v>
       </c>
       <c r="H31" s="3" t="s">
-        <v>459</v>
+        <v>457</v>
       </c>
     </row>
     <row r="32" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A32" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B32" s="5" t="s">
         <v>14</v>
@@ -11867,12 +11847,12 @@
         <v>44</v>
       </c>
       <c r="H32" s="3" t="s">
-        <v>462</v>
+        <v>460</v>
       </c>
     </row>
     <row r="33" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A33" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B33" s="5" t="s">
         <v>14</v>
@@ -11898,7 +11878,7 @@
     </row>
     <row r="34" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A34" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B34" s="5" t="s">
         <v>14</v>
@@ -11924,7 +11904,7 @@
     </row>
     <row r="35" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A35" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B35" s="5" t="s">
         <v>14</v>
@@ -11950,7 +11930,7 @@
     </row>
     <row r="36" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A36" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B36" s="5" t="s">
         <v>14</v>
@@ -11976,7 +11956,7 @@
     </row>
     <row r="37" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A37" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B37" s="5" t="s">
         <v>14</v>
@@ -11997,12 +11977,12 @@
         <v>54</v>
       </c>
       <c r="H37" s="3" t="s">
-        <v>354</v>
+        <v>353</v>
       </c>
     </row>
     <row r="38" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A38" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B38" s="5" t="s">
         <v>14</v>
@@ -12028,7 +12008,7 @@
     </row>
     <row r="39" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A39" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>14</v>
@@ -12054,7 +12034,7 @@
     </row>
     <row r="40" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A40" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B40" s="5" t="s">
         <v>14</v>
@@ -12075,12 +12055,12 @@
         <v>60</v>
       </c>
       <c r="H40" s="3" t="s">
-        <v>458</v>
+        <v>456</v>
       </c>
     </row>
     <row r="41" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A41" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B41" s="5" t="s">
         <v>14</v>
@@ -12106,7 +12086,7 @@
     </row>
     <row r="42" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A42" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B42" s="5" t="s">
         <v>14</v>
@@ -12132,7 +12112,7 @@
     </row>
     <row r="43" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A43" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B43" s="5" t="s">
         <v>14</v>
@@ -12158,7 +12138,7 @@
     </row>
     <row r="44" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A44" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B44" s="5" t="s">
         <v>14</v>
@@ -12184,7 +12164,7 @@
     </row>
     <row r="45" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A45" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B45" s="5" t="s">
         <v>14</v>
@@ -12210,7 +12190,7 @@
     </row>
     <row r="46" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A46" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B46" s="5" t="s">
         <v>14</v>
@@ -12236,7 +12216,7 @@
     </row>
     <row r="47" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A47" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B47" s="5" t="s">
         <v>14</v>
@@ -12262,7 +12242,7 @@
     </row>
     <row r="48" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A48" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B48" s="5" t="s">
         <v>14</v>
@@ -12288,7 +12268,7 @@
     </row>
     <row r="49" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A49" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B49" s="5" t="s">
         <v>14</v>
@@ -12314,7 +12294,7 @@
     </row>
     <row r="50" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A50" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B50" s="5" t="s">
         <v>14</v>
@@ -12340,7 +12320,7 @@
     </row>
     <row r="51" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A51" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B51" s="5" t="s">
         <v>14</v>
@@ -12361,12 +12341,12 @@
         <v>82</v>
       </c>
       <c r="H51" s="3" t="s">
-        <v>457</v>
+        <v>455</v>
       </c>
     </row>
     <row r="52" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A52" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B52" s="5" t="s">
         <v>14</v>
@@ -12392,7 +12372,7 @@
     </row>
     <row r="53" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A53" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B53" s="5" t="s">
         <v>14</v>
@@ -12418,7 +12398,7 @@
     </row>
     <row r="54" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A54" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B54" s="5" t="s">
         <v>14</v>
@@ -12444,7 +12424,7 @@
     </row>
     <row r="55" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A55" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B55" s="5" t="s">
         <v>14</v>
@@ -12465,12 +12445,12 @@
         <v>90</v>
       </c>
       <c r="H55" s="3" t="s">
-        <v>455</v>
+        <v>453</v>
       </c>
     </row>
     <row r="56" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A56" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B56" s="5" t="s">
         <v>14</v>
@@ -12496,7 +12476,7 @@
     </row>
     <row r="57" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A57" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B57" s="5" t="s">
         <v>14</v>
@@ -12517,12 +12497,12 @@
         <v>94</v>
       </c>
       <c r="H57" s="3" t="s">
-        <v>456</v>
+        <v>454</v>
       </c>
     </row>
     <row r="58" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A58" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B58" s="5" t="s">
         <v>14</v>
@@ -12548,7 +12528,7 @@
     </row>
     <row r="59" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A59" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B59" s="5" t="s">
         <v>14</v>
@@ -12574,7 +12554,7 @@
     </row>
     <row r="60" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A60" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B60" s="5" t="s">
         <v>14</v>
@@ -12600,7 +12580,7 @@
     </row>
     <row r="61" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A61" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B61" s="5" t="s">
         <v>14</v>
@@ -12626,7 +12606,7 @@
     </row>
     <row r="62" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A62" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B62" s="5" t="s">
         <v>14</v>
@@ -12652,7 +12632,7 @@
     </row>
     <row r="63" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A63" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B63" s="5" t="s">
         <v>14</v>
@@ -12678,7 +12658,7 @@
     </row>
     <row r="64" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A64" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B64" s="5" t="s">
         <v>107</v>
@@ -12704,7 +12684,7 @@
     </row>
     <row r="65" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A65" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B65" s="5" t="s">
         <v>107</v>
@@ -12713,24 +12693,24 @@
         <v>1</v>
       </c>
       <c r="D65" s="5" t="s">
+        <v>476</v>
+      </c>
+      <c r="E65" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F65" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G65" s="6" t="s">
+        <v>477</v>
+      </c>
+      <c r="H65" s="2" t="s">
         <v>478</v>
-      </c>
-      <c r="E65" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F65" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G65" s="6" t="s">
-        <v>479</v>
-      </c>
-      <c r="H65" s="2" t="s">
-        <v>480</v>
       </c>
     </row>
     <row r="66" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A66" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B66" s="5" t="s">
         <v>110</v>
@@ -12756,7 +12736,7 @@
     </row>
     <row r="67" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A67" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B67" s="5" t="s">
         <v>113</v>
@@ -12782,7 +12762,7 @@
     </row>
     <row r="68" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A68" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B68" s="5" t="s">
         <v>113</v>
@@ -12808,7 +12788,7 @@
     </row>
     <row r="69" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A69" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B69" s="5" t="s">
         <v>113</v>
@@ -12834,7 +12814,7 @@
     </row>
     <row r="70" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A70" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B70" s="5" t="s">
         <v>113</v>
@@ -12860,7 +12840,7 @@
     </row>
     <row r="71" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A71" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B71" s="5" t="s">
         <v>113</v>
@@ -12886,7 +12866,7 @@
     </row>
     <row r="72" spans="1:8" ht="45" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A72" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B72" s="5" t="s">
         <v>113</v>
@@ -12912,16 +12892,16 @@
     </row>
     <row r="73" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A73" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B73" s="5" t="s">
-        <v>496</v>
+        <v>494</v>
       </c>
       <c r="C73" s="5">
         <v>0</v>
       </c>
       <c r="D73" s="5" t="s">
-        <v>494</v>
+        <v>492</v>
       </c>
       <c r="E73" s="5" t="s">
         <v>8</v>
@@ -12930,15 +12910,15 @@
         <v>9</v>
       </c>
       <c r="G73" s="9" t="s">
-        <v>495</v>
+        <v>493</v>
       </c>
       <c r="H73" s="2" t="s">
-        <v>519</v>
+        <v>517</v>
       </c>
     </row>
     <row r="74" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A74" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B74" s="5" t="s">
         <v>12</v>
@@ -12964,7 +12944,7 @@
     </row>
     <row r="75" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A75" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B75" s="5" t="s">
         <v>12</v>
@@ -12990,7 +12970,7 @@
     </row>
     <row r="76" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A76" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B76" s="5" t="s">
         <v>12</v>
@@ -13016,7 +12996,7 @@
     </row>
     <row r="77" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A77" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B77" s="5" t="s">
         <v>12</v>
@@ -13042,7 +13022,7 @@
     </row>
     <row r="78" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A78" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B78" s="5" t="s">
         <v>12</v>
@@ -13068,7 +13048,7 @@
     </row>
     <row r="79" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A79" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B79" s="5" t="s">
         <v>12</v>
@@ -13094,7 +13074,7 @@
     </row>
     <row r="80" spans="1:8" ht="60" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A80" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B80" s="5" t="s">
         <v>138</v>
@@ -13120,7 +13100,7 @@
     </row>
     <row r="81" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A81" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B81" s="5" t="s">
         <v>138</v>
@@ -13146,7 +13126,7 @@
     </row>
     <row r="82" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A82" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B82" s="5" t="s">
         <v>143</v>
@@ -13167,12 +13147,12 @@
         <v>145</v>
       </c>
       <c r="H82" s="3" t="s">
-        <v>518</v>
-      </c>
-    </row>
-    <row r="83" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="83" spans="1:8" ht="162" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A83" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B83" s="5" t="s">
         <v>143</v>
@@ -13193,12 +13173,12 @@
         <v>147</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>271</v>
+        <v>528</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A84" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B84" s="5" t="s">
         <v>10</v>
@@ -13219,12 +13199,12 @@
         <v>149</v>
       </c>
       <c r="H84" s="2" t="s">
-        <v>430</v>
+        <v>429</v>
       </c>
     </row>
     <row r="85" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A85" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B85" s="5" t="s">
         <v>150</v>
@@ -13245,12 +13225,12 @@
         <v>152</v>
       </c>
       <c r="H85" s="2" t="s">
-        <v>272</v>
+        <v>271</v>
       </c>
     </row>
     <row r="86" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A86" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B86" s="5" t="s">
         <v>150</v>
@@ -13271,12 +13251,12 @@
         <v>154</v>
       </c>
       <c r="H86" s="2" t="s">
-        <v>273</v>
+        <v>272</v>
       </c>
     </row>
     <row r="87" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A87" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B87" s="5" t="s">
         <v>155</v>
@@ -13297,12 +13277,12 @@
         <v>157</v>
       </c>
       <c r="H87" s="2" t="s">
-        <v>274</v>
+        <v>273</v>
       </c>
     </row>
     <row r="88" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A88" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B88" s="5" t="s">
         <v>155</v>
@@ -13323,12 +13303,12 @@
         <v>159</v>
       </c>
       <c r="H88" s="3" t="s">
-        <v>450</v>
+        <v>448</v>
       </c>
     </row>
     <row r="89" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A89" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B89" s="5" t="s">
         <v>160</v>
@@ -13349,12 +13329,12 @@
         <v>162</v>
       </c>
       <c r="H89" s="3" t="s">
-        <v>275</v>
+        <v>274</v>
       </c>
     </row>
     <row r="90" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A90" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B90" s="5" t="s">
         <v>160</v>
@@ -13375,12 +13355,12 @@
         <v>164</v>
       </c>
       <c r="H90" s="2" t="s">
-        <v>276</v>
+        <v>275</v>
       </c>
     </row>
     <row r="91" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A91" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B91" s="5" t="s">
         <v>160</v>
@@ -13401,12 +13381,12 @@
         <v>166</v>
       </c>
       <c r="H91" s="2" t="s">
-        <v>477</v>
+        <v>475</v>
       </c>
     </row>
     <row r="92" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A92" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B92" s="5" t="s">
         <v>160</v>
@@ -13427,12 +13407,12 @@
         <v>168</v>
       </c>
       <c r="H92" s="3" t="s">
-        <v>277</v>
+        <v>276</v>
       </c>
     </row>
     <row r="93" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A93" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B93" s="5" t="s">
         <v>160</v>
@@ -13453,12 +13433,12 @@
         <v>170</v>
       </c>
       <c r="H93" s="3" t="s">
-        <v>467</v>
+        <v>465</v>
       </c>
     </row>
     <row r="94" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A94" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B94" s="5" t="s">
         <v>171</v>
@@ -13479,12 +13459,12 @@
         <v>173</v>
       </c>
       <c r="H94" s="2" t="s">
-        <v>473</v>
+        <v>471</v>
       </c>
     </row>
     <row r="95" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A95" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B95" s="5" t="s">
         <v>171</v>
@@ -13505,12 +13485,12 @@
         <v>175</v>
       </c>
       <c r="H95" s="3" t="s">
-        <v>451</v>
+        <v>449</v>
       </c>
     </row>
     <row r="96" spans="1:8" ht="304.2" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A96" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B96" s="5" t="s">
         <v>11</v>
@@ -13528,15 +13508,15 @@
         <v>9</v>
       </c>
       <c r="G96" s="6" t="s">
-        <v>365</v>
+        <v>364</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A97" s="5" t="s">
-        <v>485</v>
+        <v>483</v>
       </c>
       <c r="B97" s="5" t="s">
         <v>10</v>
@@ -13545,24 +13525,24 @@
         <v>1</v>
       </c>
       <c r="D97" s="5" t="s">
+        <v>484</v>
+      </c>
+      <c r="E97" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F97" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G97" s="6" t="s">
         <v>486</v>
       </c>
-      <c r="E97" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F97" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G97" s="6" t="s">
-        <v>488</v>
-      </c>
       <c r="H97" s="2" t="s">
-        <v>487</v>
+        <v>485</v>
       </c>
     </row>
     <row r="98" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A98" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B98" s="5" t="s">
         <v>11</v>
@@ -13583,12 +13563,12 @@
         <v>178</v>
       </c>
       <c r="H98" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="99" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A99" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B99" s="5" t="s">
         <v>179</v>
@@ -13609,12 +13589,12 @@
         <v>181</v>
       </c>
       <c r="H99" s="2" t="s">
-        <v>279</v>
+        <v>278</v>
       </c>
     </row>
     <row r="100" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A100" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B100" s="5" t="s">
         <v>179</v>
@@ -13635,12 +13615,12 @@
         <v>183</v>
       </c>
       <c r="H100" s="3" t="s">
-        <v>452</v>
+        <v>450</v>
       </c>
     </row>
     <row r="101" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A101" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B101" s="5" t="s">
         <v>184</v>
@@ -13661,12 +13641,12 @@
         <v>186</v>
       </c>
       <c r="H101" s="3" t="s">
-        <v>280</v>
+        <v>279</v>
       </c>
     </row>
     <row r="102" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A102" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B102" s="5" t="s">
         <v>184</v>
@@ -13687,12 +13667,12 @@
         <v>188</v>
       </c>
       <c r="H102" s="3" t="s">
-        <v>281</v>
+        <v>280</v>
       </c>
     </row>
     <row r="103" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A103" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B103" s="5" t="s">
         <v>184</v>
@@ -13713,12 +13693,12 @@
         <v>190</v>
       </c>
       <c r="H103" s="3" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
     </row>
     <row r="104" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A104" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B104" s="5" t="s">
         <v>184</v>
@@ -13739,12 +13719,12 @@
         <v>192</v>
       </c>
       <c r="H104" s="2" t="s">
-        <v>283</v>
+        <v>282</v>
       </c>
     </row>
     <row r="105" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A105" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B105" s="5" t="s">
         <v>184</v>
@@ -13765,12 +13745,12 @@
         <v>194</v>
       </c>
       <c r="H105" s="3" t="s">
-        <v>284</v>
+        <v>283</v>
       </c>
     </row>
     <row r="106" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A106" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B106" s="5" t="s">
         <v>184</v>
@@ -13791,12 +13771,12 @@
         <v>196</v>
       </c>
       <c r="H106" s="3" t="s">
-        <v>285</v>
+        <v>284</v>
       </c>
     </row>
     <row r="107" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A107" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B107" s="5" t="s">
         <v>197</v>
@@ -13817,12 +13797,12 @@
         <v>199</v>
       </c>
       <c r="H107" s="3" t="s">
-        <v>286</v>
+        <v>285</v>
       </c>
     </row>
     <row r="108" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A108" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B108" s="5" t="s">
         <v>197</v>
@@ -13843,12 +13823,12 @@
         <v>201</v>
       </c>
       <c r="H108" s="3" t="s">
-        <v>287</v>
+        <v>286</v>
       </c>
     </row>
     <row r="109" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A109" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B109" s="5" t="s">
         <v>202</v>
@@ -13866,15 +13846,15 @@
         <v>9</v>
       </c>
       <c r="G109" s="6" t="s">
-        <v>470</v>
+        <v>468</v>
       </c>
       <c r="H109" s="3" t="s">
-        <v>469</v>
+        <v>467</v>
       </c>
     </row>
     <row r="110" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A110" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B110" s="5" t="s">
         <v>202</v>
@@ -13892,15 +13872,15 @@
         <v>9</v>
       </c>
       <c r="G110" s="6" t="s">
-        <v>348</v>
+        <v>347</v>
       </c>
       <c r="H110" s="2" t="s">
-        <v>489</v>
+        <v>487</v>
       </c>
     </row>
     <row r="111" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A111" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B111" s="5" t="s">
         <v>205</v>
@@ -13918,15 +13898,15 @@
         <v>9</v>
       </c>
       <c r="G111" s="6" t="s">
-        <v>468</v>
+        <v>466</v>
       </c>
       <c r="H111" s="3" t="s">
-        <v>474</v>
+        <v>472</v>
       </c>
     </row>
     <row r="112" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A112" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B112" s="5" t="s">
         <v>207</v>
@@ -13944,7 +13924,7 @@
         <v>9</v>
       </c>
       <c r="G112" s="6" t="s">
-        <v>475</v>
+        <v>473</v>
       </c>
       <c r="H112" s="3" t="s">
         <v>260</v>
@@ -13952,7 +13932,7 @@
     </row>
     <row r="113" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A113" s="5" t="s">
-        <v>364</v>
+        <v>363</v>
       </c>
       <c r="B113" s="5" t="s">
         <v>209</v>
@@ -13970,7 +13950,7 @@
         <v>9</v>
       </c>
       <c r="G113" s="6" t="s">
-        <v>476</v>
+        <v>474</v>
       </c>
       <c r="H113" s="3" t="s">
         <v>261</v>
@@ -13978,7 +13958,7 @@
     </row>
     <row r="114" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A114" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B114" s="5" t="s">
         <v>211</v>
@@ -13996,15 +13976,15 @@
         <v>9</v>
       </c>
       <c r="G114" s="6" t="s">
+        <v>355</v>
+      </c>
+      <c r="H114" s="3" t="s">
         <v>356</v>
-      </c>
-      <c r="H114" s="3" t="s">
-        <v>357</v>
       </c>
     </row>
     <row r="115" spans="1:8" ht="43.2" x14ac:dyDescent="0.3">
       <c r="A115" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B115" s="5" t="s">
         <v>211</v>
@@ -14025,12 +14005,12 @@
         <v>214</v>
       </c>
       <c r="H115" s="3" t="s">
-        <v>358</v>
+        <v>357</v>
       </c>
     </row>
     <row r="116" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A116" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B116" s="5" t="s">
         <v>215</v>
@@ -14051,12 +14031,12 @@
         <v>217</v>
       </c>
       <c r="H116" s="2" t="s">
-        <v>347</v>
+        <v>346</v>
       </c>
     </row>
     <row r="117" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A117" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B117" s="5" t="s">
         <v>218</v>
@@ -14077,12 +14057,12 @@
         <v>220</v>
       </c>
       <c r="H117" s="3" t="s">
-        <v>346</v>
+        <v>345</v>
       </c>
     </row>
     <row r="118" spans="1:8" ht="115.2" x14ac:dyDescent="0.3">
       <c r="A118" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B118" s="5" t="s">
         <v>218</v>
@@ -14091,362 +14071,362 @@
         <v>1</v>
       </c>
       <c r="D118" s="5" t="s">
+        <v>511</v>
+      </c>
+      <c r="E118" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F118" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G118" s="6" t="s">
+        <v>512</v>
+      </c>
+      <c r="H118" s="3" t="s">
         <v>513</v>
-      </c>
-      <c r="E118" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F118" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G118" s="6" t="s">
-        <v>514</v>
-      </c>
-      <c r="H118" s="3" t="s">
-        <v>515</v>
       </c>
     </row>
     <row r="119" spans="1:8" ht="165" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A119" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B119" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C119" s="5">
         <v>0</v>
       </c>
       <c r="D119" s="5" t="s">
+        <v>369</v>
+      </c>
+      <c r="E119" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F119" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G119" s="6" t="s">
         <v>370</v>
       </c>
-      <c r="E119" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F119" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G119" s="6" t="s">
-        <v>371</v>
-      </c>
       <c r="H119" s="2" t="s">
-        <v>517</v>
+        <v>515</v>
       </c>
     </row>
     <row r="120" spans="1:8" ht="225" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A120" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B120" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C120" s="5">
         <v>1</v>
       </c>
       <c r="D120" s="5" t="s">
+        <v>371</v>
+      </c>
+      <c r="E120" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F120" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G120" s="6" t="s">
         <v>372</v>
       </c>
-      <c r="E120" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F120" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G120" s="6" t="s">
-        <v>373</v>
-      </c>
       <c r="H120" s="2" t="s">
-        <v>516</v>
+        <v>514</v>
       </c>
     </row>
     <row r="121" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A121" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B121" s="5" t="s">
-        <v>291</v>
+        <v>290</v>
       </c>
       <c r="C121" s="5">
         <v>2</v>
       </c>
       <c r="D121" s="5" t="s">
+        <v>291</v>
+      </c>
+      <c r="E121" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F121" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G121" s="6" t="s">
         <v>292</v>
       </c>
-      <c r="E121" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F121" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G121" s="6" t="s">
-        <v>293</v>
-      </c>
       <c r="H121" s="2" t="s">
-        <v>521</v>
+        <v>519</v>
       </c>
     </row>
     <row r="122" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A122" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B122" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C122" s="5">
         <v>0</v>
       </c>
       <c r="D122" s="5" t="s">
+        <v>294</v>
+      </c>
+      <c r="E122" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F122" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G122" s="6" t="s">
         <v>295</v>
       </c>
-      <c r="E122" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F122" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G122" s="6" t="s">
+      <c r="H122" s="3" t="s">
         <v>296</v>
-      </c>
-      <c r="H122" s="3" t="s">
-        <v>297</v>
       </c>
     </row>
     <row r="123" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A123" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B123" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C123" s="5">
         <v>1</v>
       </c>
       <c r="D123" s="5" t="s">
+        <v>297</v>
+      </c>
+      <c r="E123" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F123" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G123" s="6" t="s">
         <v>298</v>
       </c>
-      <c r="E123" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F123" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G123" s="6" t="s">
-        <v>299</v>
-      </c>
       <c r="H123" s="3" t="s">
-        <v>520</v>
+        <v>518</v>
       </c>
     </row>
     <row r="124" spans="1:8" ht="90" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A124" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B124" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C124" s="5">
         <v>2</v>
       </c>
       <c r="D124" s="5" t="s">
+        <v>299</v>
+      </c>
+      <c r="E124" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F124" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G124" s="6" t="s">
         <v>300</v>
       </c>
-      <c r="E124" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F124" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G124" s="6" t="s">
-        <v>301</v>
-      </c>
       <c r="H124" s="2" t="s">
-        <v>522</v>
+        <v>520</v>
       </c>
     </row>
     <row r="125" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A125" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B125" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C125" s="5">
         <v>3</v>
       </c>
       <c r="D125" s="5" t="s">
+        <v>301</v>
+      </c>
+      <c r="E125" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F125" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G125" s="6" t="s">
         <v>302</v>
       </c>
-      <c r="E125" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F125" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G125" s="6" t="s">
-        <v>303</v>
-      </c>
       <c r="H125" s="3" t="s">
-        <v>523</v>
+        <v>521</v>
       </c>
     </row>
     <row r="126" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A126" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B126" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C126" s="5">
         <v>4</v>
       </c>
       <c r="D126" s="5" t="s">
+        <v>303</v>
+      </c>
+      <c r="E126" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F126" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G126" s="6" t="s">
         <v>304</v>
       </c>
-      <c r="E126" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F126" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G126" s="6" t="s">
+      <c r="H126" s="3" t="s">
         <v>305</v>
-      </c>
-      <c r="H126" s="3" t="s">
-        <v>306</v>
       </c>
     </row>
     <row r="127" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A127" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B127" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C127" s="5">
         <v>5</v>
       </c>
       <c r="D127" s="5" t="s">
+        <v>306</v>
+      </c>
+      <c r="E127" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F127" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G127" s="6" t="s">
         <v>307</v>
       </c>
-      <c r="E127" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F127" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G127" s="6" t="s">
-        <v>308</v>
-      </c>
       <c r="H127" s="3" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
     </row>
     <row r="128" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A128" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B128" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C128" s="5">
         <v>6</v>
       </c>
       <c r="D128" s="5" t="s">
+        <v>308</v>
+      </c>
+      <c r="E128" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F128" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G128" s="6" t="s">
         <v>309</v>
       </c>
-      <c r="E128" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F128" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G128" s="6" t="s">
+      <c r="H128" s="2" t="s">
         <v>310</v>
-      </c>
-      <c r="H128" s="2" t="s">
-        <v>311</v>
       </c>
     </row>
     <row r="129" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A129" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B129" s="5" t="s">
-        <v>294</v>
+        <v>293</v>
       </c>
       <c r="C129" s="5">
         <v>7</v>
       </c>
       <c r="D129" s="5" t="s">
+        <v>311</v>
+      </c>
+      <c r="E129" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F129" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G129" s="6" t="s">
         <v>312</v>
       </c>
-      <c r="E129" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F129" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G129" s="6" t="s">
+      <c r="H129" s="2" t="s">
         <v>313</v>
-      </c>
-      <c r="H129" s="2" t="s">
-        <v>314</v>
       </c>
     </row>
     <row r="130" spans="1:8" ht="390" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A130" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B130" s="5" t="s">
-        <v>315</v>
+        <v>314</v>
       </c>
       <c r="C130" s="5">
         <v>0</v>
       </c>
       <c r="D130" s="5" t="s">
+        <v>315</v>
+      </c>
+      <c r="E130" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F130" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G130" s="6" t="s">
         <v>316</v>
       </c>
-      <c r="E130" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F130" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G130" s="6" t="s">
-        <v>317</v>
-      </c>
       <c r="H130" s="6" t="s">
-        <v>317</v>
+        <v>316</v>
       </c>
     </row>
     <row r="131" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A131" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B131" s="5" t="s">
-        <v>318</v>
+        <v>317</v>
       </c>
       <c r="C131" s="5">
         <v>0</v>
       </c>
       <c r="D131" s="5" t="s">
+        <v>318</v>
+      </c>
+      <c r="E131" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F131" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G131" s="6" t="s">
         <v>319</v>
       </c>
-      <c r="E131" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F131" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G131" s="6" t="s">
-        <v>320</v>
-      </c>
       <c r="H131" s="3" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
     </row>
     <row r="132" spans="1:8" ht="30" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A132" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B132" s="5" t="s">
         <v>11</v>
@@ -14455,24 +14435,24 @@
         <v>0</v>
       </c>
       <c r="D132" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="E132" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F132" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G132" s="6" t="s">
         <v>321</v>
       </c>
-      <c r="E132" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F132" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G132" s="6" t="s">
+      <c r="H132" s="2" t="s">
         <v>322</v>
-      </c>
-      <c r="H132" s="2" t="s">
-        <v>323</v>
       </c>
     </row>
     <row r="133" spans="1:8" ht="230.4" x14ac:dyDescent="0.3">
       <c r="A133" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B133" s="5" t="s">
         <v>11</v>
@@ -14481,7 +14461,7 @@
         <v>1</v>
       </c>
       <c r="D133" s="5" t="s">
-        <v>471</v>
+        <v>469</v>
       </c>
       <c r="E133" s="5" t="s">
         <v>8</v>
@@ -14490,15 +14470,15 @@
         <v>9</v>
       </c>
       <c r="G133" s="6" t="s">
-        <v>472</v>
+        <v>470</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A134" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B134" s="5" t="s">
         <v>11</v>
@@ -14507,24 +14487,24 @@
         <v>2</v>
       </c>
       <c r="D134" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="E134" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F134" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G134" s="6" t="s">
         <v>324</v>
       </c>
-      <c r="E134" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F134" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G134" s="6" t="s">
+      <c r="H134" s="2" t="s">
         <v>325</v>
-      </c>
-      <c r="H134" s="2" t="s">
-        <v>326</v>
       </c>
     </row>
     <row r="135" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A135" s="5" t="s">
-        <v>367</v>
+        <v>366</v>
       </c>
       <c r="B135" s="5" t="s">
         <v>11</v>
@@ -14545,192 +14525,192 @@
         <v>178</v>
       </c>
       <c r="H135" s="3" t="s">
-        <v>278</v>
+        <v>277</v>
       </c>
     </row>
     <row r="136" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A136" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B136" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C136" s="5">
         <v>0</v>
       </c>
       <c r="D136" s="5" t="s">
+        <v>379</v>
+      </c>
+      <c r="E136" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F136" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G136" s="6" t="s">
         <v>380</v>
       </c>
-      <c r="E136" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F136" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G136" s="6" t="s">
-        <v>381</v>
-      </c>
       <c r="H136" s="8" t="s">
-        <v>442</v>
+        <v>441</v>
       </c>
     </row>
     <row r="137" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A137" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B137" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C137" s="5">
         <v>1</v>
       </c>
       <c r="D137" s="5" t="s">
+        <v>381</v>
+      </c>
+      <c r="E137" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F137" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G137" s="6" t="s">
         <v>382</v>
       </c>
-      <c r="E137" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F137" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G137" s="6" t="s">
-        <v>383</v>
-      </c>
       <c r="H137" s="2" t="s">
-        <v>439</v>
+        <v>438</v>
       </c>
     </row>
     <row r="138" spans="1:8" ht="188.4" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A138" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B138" s="5" t="s">
-        <v>379</v>
+        <v>378</v>
       </c>
       <c r="C138" s="5">
         <v>2</v>
       </c>
       <c r="D138" s="5" t="s">
+        <v>383</v>
+      </c>
+      <c r="E138" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F138" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G138" s="6" t="s">
         <v>384</v>
       </c>
-      <c r="E138" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F138" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G138" s="6" t="s">
-        <v>385</v>
-      </c>
       <c r="H138" s="2" t="s">
-        <v>441</v>
+        <v>440</v>
       </c>
     </row>
     <row r="139" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A139" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B139" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C139" s="5">
         <v>0</v>
       </c>
       <c r="D139" s="5" t="s">
+        <v>385</v>
+      </c>
+      <c r="E139" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F139" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G139" s="6" t="s">
         <v>386</v>
-      </c>
-      <c r="E139" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F139" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G139" s="6" t="s">
-        <v>387</v>
       </c>
       <c r="H139" s="7"/>
     </row>
     <row r="140" spans="1:8" ht="105" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A140" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B140" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C140" s="5">
         <v>1</v>
       </c>
       <c r="D140" s="5" t="s">
+        <v>387</v>
+      </c>
+      <c r="E140" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F140" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G140" s="6" t="s">
         <v>388</v>
       </c>
-      <c r="E140" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F140" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G140" s="6" t="s">
-        <v>389</v>
-      </c>
       <c r="H140" s="2" t="s">
-        <v>437</v>
+        <v>436</v>
       </c>
     </row>
     <row r="141" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A141" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B141" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C141" s="5">
         <v>2</v>
       </c>
       <c r="D141" s="5" t="s">
+        <v>389</v>
+      </c>
+      <c r="E141" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F141" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G141" s="6" t="s">
         <v>390</v>
       </c>
-      <c r="E141" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F141" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G141" s="6" t="s">
-        <v>391</v>
-      </c>
       <c r="H141" s="2" t="s">
-        <v>453</v>
+        <v>451</v>
       </c>
     </row>
     <row r="142" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A142" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B142" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C142" s="5">
         <v>3</v>
       </c>
       <c r="D142" s="5" t="s">
+        <v>391</v>
+      </c>
+      <c r="E142" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F142" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G142" s="6" t="s">
         <v>392</v>
       </c>
-      <c r="E142" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F142" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G142" s="6" t="s">
-        <v>393</v>
-      </c>
       <c r="H142" s="2" t="s">
-        <v>454</v>
+        <v>452</v>
       </c>
     </row>
     <row r="143" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A143" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B143" s="5" t="s">
         <v>171</v>
@@ -14739,22 +14719,22 @@
         <v>0</v>
       </c>
       <c r="D143" s="5" t="s">
+        <v>393</v>
+      </c>
+      <c r="E143" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F143" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G143" s="6" t="s">
         <v>394</v>
-      </c>
-      <c r="E143" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F143" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G143" s="6" t="s">
-        <v>395</v>
       </c>
       <c r="H143" s="7"/>
     </row>
     <row r="144" spans="1:8" ht="100.8" x14ac:dyDescent="0.3">
       <c r="A144" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B144" s="5" t="s">
         <v>171</v>
@@ -14763,24 +14743,24 @@
         <v>1</v>
       </c>
       <c r="D144" s="5" t="s">
+        <v>395</v>
+      </c>
+      <c r="E144" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F144" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G144" s="6" t="s">
         <v>396</v>
       </c>
-      <c r="E144" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F144" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G144" s="6" t="s">
-        <v>397</v>
-      </c>
       <c r="H144" s="2" t="s">
-        <v>438</v>
+        <v>437</v>
       </c>
     </row>
     <row r="145" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A145" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B145" s="5" t="s">
         <v>171</v>
@@ -14789,24 +14769,24 @@
         <v>2</v>
       </c>
       <c r="D145" s="5" t="s">
+        <v>397</v>
+      </c>
+      <c r="E145" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F145" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G145" s="6" t="s">
         <v>398</v>
       </c>
-      <c r="E145" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F145" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G145" s="6" t="s">
-        <v>399</v>
-      </c>
       <c r="H145" s="2" t="s">
-        <v>429</v>
+        <v>428</v>
       </c>
     </row>
     <row r="146" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A146" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B146" s="5" t="s">
         <v>171</v>
@@ -14815,24 +14795,24 @@
         <v>3</v>
       </c>
       <c r="D146" s="5" t="s">
+        <v>399</v>
+      </c>
+      <c r="E146" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F146" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G146" s="6" t="s">
         <v>400</v>
       </c>
-      <c r="E146" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F146" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G146" s="6" t="s">
-        <v>401</v>
-      </c>
       <c r="H146" s="2" t="s">
-        <v>427</v>
+        <v>426</v>
       </c>
     </row>
     <row r="147" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A147" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B147" s="5" t="s">
         <v>171</v>
@@ -14841,369 +14821,369 @@
         <v>4</v>
       </c>
       <c r="D147" s="5" t="s">
+        <v>401</v>
+      </c>
+      <c r="E147" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F147" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G147" s="6" t="s">
         <v>402</v>
       </c>
-      <c r="E147" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F147" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G147" s="6" t="s">
-        <v>403</v>
-      </c>
       <c r="H147" s="2" t="s">
-        <v>428</v>
+        <v>427</v>
       </c>
     </row>
     <row r="148" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A148" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B148" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C148" s="5">
         <v>0</v>
       </c>
       <c r="D148" s="5" t="s">
+        <v>404</v>
+      </c>
+      <c r="E148" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F148" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G148" s="6" t="s">
         <v>405</v>
-      </c>
-      <c r="E148" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F148" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G148" s="6" t="s">
-        <v>406</v>
       </c>
       <c r="H148" s="7"/>
     </row>
     <row r="149" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A149" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B149" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C149" s="5">
         <v>1</v>
       </c>
       <c r="D149" s="5" t="s">
+        <v>406</v>
+      </c>
+      <c r="E149" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F149" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G149" s="6" t="s">
         <v>407</v>
       </c>
-      <c r="E149" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F149" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G149" s="6" t="s">
-        <v>408</v>
-      </c>
       <c r="H149" s="2" t="s">
-        <v>440</v>
+        <v>439</v>
       </c>
     </row>
     <row r="150" spans="1:8" ht="187.2" x14ac:dyDescent="0.3">
       <c r="A150" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B150" s="5" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C150" s="5">
         <v>2</v>
       </c>
       <c r="D150" s="5" t="s">
+        <v>408</v>
+      </c>
+      <c r="E150" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F150" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G150" s="6" t="s">
         <v>409</v>
       </c>
-      <c r="E150" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F150" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G150" s="6" t="s">
-        <v>410</v>
-      </c>
       <c r="H150" s="2" t="s">
-        <v>443</v>
+        <v>442</v>
       </c>
     </row>
     <row r="151" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A151" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B151" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C151" s="5">
         <v>0</v>
       </c>
       <c r="D151" s="5" t="s">
+        <v>411</v>
+      </c>
+      <c r="E151" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F151" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G151" s="6" t="s">
         <v>412</v>
       </c>
-      <c r="E151" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F151" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G151" s="6" t="s">
-        <v>413</v>
-      </c>
       <c r="H151" s="2" t="s">
-        <v>436</v>
+        <v>435</v>
       </c>
     </row>
     <row r="152" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A152" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B152" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C152" s="5">
         <v>1</v>
       </c>
       <c r="D152" s="5" t="s">
+        <v>413</v>
+      </c>
+      <c r="E152" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F152" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G152" s="6" t="s">
         <v>414</v>
       </c>
-      <c r="E152" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F152" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G152" s="6" t="s">
-        <v>415</v>
-      </c>
       <c r="H152" s="2" t="s">
-        <v>435</v>
+        <v>434</v>
       </c>
     </row>
     <row r="153" spans="1:8" ht="57.6" x14ac:dyDescent="0.3">
       <c r="A153" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B153" s="5" t="s">
-        <v>411</v>
+        <v>410</v>
       </c>
       <c r="C153" s="5">
         <v>2</v>
       </c>
       <c r="D153" s="5" t="s">
+        <v>415</v>
+      </c>
+      <c r="E153" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F153" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G153" s="6" t="s">
         <v>416</v>
       </c>
-      <c r="E153" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F153" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G153" s="6" t="s">
-        <v>417</v>
-      </c>
       <c r="H153" s="2" t="s">
-        <v>434</v>
+        <v>433</v>
       </c>
     </row>
     <row r="154" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A154" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B154" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C154" s="5">
         <v>0</v>
       </c>
       <c r="D154" s="5" t="s">
+        <v>417</v>
+      </c>
+      <c r="E154" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F154" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G154" s="6" t="s">
         <v>418</v>
       </c>
-      <c r="E154" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F154" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G154" s="6" t="s">
-        <v>419</v>
-      </c>
       <c r="H154" s="2" t="s">
-        <v>433</v>
+        <v>432</v>
       </c>
     </row>
     <row r="155" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A155" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B155" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C155" s="5">
         <v>1</v>
       </c>
       <c r="D155" s="5" t="s">
+        <v>419</v>
+      </c>
+      <c r="E155" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F155" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G155" s="6" t="s">
         <v>420</v>
       </c>
-      <c r="E155" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F155" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G155" s="6" t="s">
-        <v>421</v>
-      </c>
       <c r="H155" s="2" t="s">
-        <v>432</v>
+        <v>431</v>
       </c>
     </row>
     <row r="156" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A156" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B156" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C156" s="5">
         <v>2</v>
       </c>
       <c r="D156" s="5" t="s">
+        <v>421</v>
+      </c>
+      <c r="E156" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F156" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G156" s="6" t="s">
         <v>422</v>
       </c>
-      <c r="E156" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F156" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G156" s="6" t="s">
-        <v>423</v>
-      </c>
       <c r="H156" s="2" t="s">
-        <v>431</v>
+        <v>430</v>
       </c>
     </row>
     <row r="157" spans="1:8" ht="72" x14ac:dyDescent="0.3">
       <c r="A157" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B157" s="5" t="s">
-        <v>424</v>
+        <v>423</v>
       </c>
       <c r="C157" s="5">
         <v>0</v>
       </c>
       <c r="D157" s="5" t="s">
+        <v>424</v>
+      </c>
+      <c r="E157" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F157" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G157" s="6" t="s">
         <v>425</v>
       </c>
-      <c r="E157" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F157" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G157" s="6" t="s">
-        <v>426</v>
-      </c>
       <c r="H157" s="2" t="s">
-        <v>426</v>
+        <v>425</v>
       </c>
     </row>
     <row r="158" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A158" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B158" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C158" s="5">
         <v>0</v>
       </c>
       <c r="D158" s="5" t="s">
+        <v>376</v>
+      </c>
+      <c r="E158" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F158" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G158" s="6" t="s">
         <v>377</v>
       </c>
-      <c r="E158" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F158" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G158" s="6" t="s">
-        <v>378</v>
-      </c>
       <c r="H158" s="3" t="s">
-        <v>328</v>
+        <v>327</v>
       </c>
     </row>
     <row r="159" spans="1:8" ht="144" x14ac:dyDescent="0.3">
       <c r="A159" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B159" s="5" t="s">
-        <v>327</v>
+        <v>326</v>
       </c>
       <c r="C159" s="5">
         <v>1</v>
       </c>
       <c r="D159" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="E159" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F159" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G159" s="6" t="s">
         <v>329</v>
       </c>
-      <c r="E159" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F159" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G159" s="6" t="s">
-        <v>330</v>
-      </c>
       <c r="H159" s="2" t="s">
-        <v>374</v>
+        <v>373</v>
       </c>
     </row>
     <row r="160" spans="1:8" ht="86.4" x14ac:dyDescent="0.3">
       <c r="A160" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B160" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C160" s="5">
         <v>0</v>
       </c>
       <c r="D160" s="5" t="s">
+        <v>331</v>
+      </c>
+      <c r="E160" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F160" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G160" s="6" t="s">
         <v>332</v>
       </c>
-      <c r="E160" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F160" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G160" s="6" t="s">
-        <v>333</v>
-      </c>
       <c r="H160" s="2" t="s">
-        <v>369</v>
+        <v>368</v>
       </c>
     </row>
     <row r="161" spans="1:8" ht="409.6" x14ac:dyDescent="0.3">
       <c r="A161" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B161" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C161" s="5">
         <v>1</v>
       </c>
       <c r="D161" s="5" t="s">
-        <v>334</v>
+        <v>333</v>
       </c>
       <c r="E161" s="5" t="s">
         <v>8</v>
@@ -15212,24 +15192,24 @@
         <v>9</v>
       </c>
       <c r="G161" s="6" t="s">
-        <v>375</v>
+        <v>374</v>
       </c>
       <c r="H161" s="2" t="s">
-        <v>446</v>
+        <v>527</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A162" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B162" s="5" t="s">
-        <v>331</v>
+        <v>330</v>
       </c>
       <c r="C162" s="5">
         <v>2</v>
       </c>
       <c r="D162" s="5" t="s">
-        <v>335</v>
+        <v>334</v>
       </c>
       <c r="E162" s="5" t="s">
         <v>8</v>
@@ -15238,93 +15218,93 @@
         <v>9</v>
       </c>
       <c r="G162" s="6" t="s">
+        <v>443</v>
+      </c>
+      <c r="H162" s="2" t="s">
         <v>444</v>
-      </c>
-      <c r="H162" s="2" t="s">
-        <v>445</v>
       </c>
     </row>
     <row r="163" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A163" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B163" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C163" s="5">
         <v>0</v>
       </c>
       <c r="D163" s="5" t="s">
+        <v>336</v>
+      </c>
+      <c r="E163" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F163" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G163" s="6" t="s">
         <v>337</v>
       </c>
-      <c r="E163" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F163" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G163" s="6" t="s">
+      <c r="H163" s="2" t="s">
         <v>338</v>
-      </c>
-      <c r="H163" s="2" t="s">
-        <v>339</v>
       </c>
     </row>
     <row r="164" spans="1:8" ht="28.8" x14ac:dyDescent="0.3">
       <c r="A164" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B164" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C164" s="5">
         <v>1</v>
       </c>
       <c r="D164" s="5" t="s">
+        <v>339</v>
+      </c>
+      <c r="E164" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F164" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G164" s="6" t="s">
         <v>340</v>
       </c>
-      <c r="E164" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F164" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G164" s="6" t="s">
+      <c r="H164" s="3" t="s">
         <v>341</v>
-      </c>
-      <c r="H164" s="3" t="s">
-        <v>342</v>
       </c>
     </row>
     <row r="165" spans="1:8" x14ac:dyDescent="0.3">
       <c r="A165" s="5" t="s">
-        <v>368</v>
+        <v>367</v>
       </c>
       <c r="B165" s="5" t="s">
-        <v>336</v>
+        <v>335</v>
       </c>
       <c r="C165" s="5">
         <v>2</v>
       </c>
       <c r="D165" s="5" t="s">
+        <v>342</v>
+      </c>
+      <c r="E165" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F165" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G165" s="6" t="s">
         <v>343</v>
       </c>
-      <c r="E165" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F165" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G165" s="6" t="s">
+      <c r="H165" s="3" t="s">
         <v>344</v>
-      </c>
-      <c r="H165" s="3" t="s">
-        <v>345</v>
       </c>
     </row>
     <row r="166" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
       <c r="A166" s="5" t="s">
-        <v>366</v>
+        <v>365</v>
       </c>
       <c r="B166" s="5" t="s">
         <v>215</v>
@@ -15333,19 +15313,19 @@
         <v>1</v>
       </c>
       <c r="D166" s="5" t="s">
+        <v>445</v>
+      </c>
+      <c r="E166" s="5" t="s">
+        <v>8</v>
+      </c>
+      <c r="F166" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="G166" s="6" t="s">
+        <v>446</v>
+      </c>
+      <c r="H166" s="2" t="s">
         <v>447</v>
-      </c>
-      <c r="E166" s="5" t="s">
-        <v>8</v>
-      </c>
-      <c r="F166" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G166" s="6" t="s">
-        <v>448</v>
-      </c>
-      <c r="H166" s="2" t="s">
-        <v>449</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
load saved answers page translated
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,14 +8,15 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{623215B1-0F92-4197-9BCF-ECBEC70D26C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4E1BBD-C5A1-45D0-A20A-113D6283100E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-37500" yWindow="-3855" windowWidth="23010" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-36270" yWindow="-3630" windowWidth="32625" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>

</xml_diff>

<commit_message>
Spanish url arg vars defined
</commit_message>
<xml_diff>
--- a/docassemble/ILAO/data/sources/ILAO_es.xlsx
+++ b/docassemble/ILAO/data/sources/ILAO_es.xlsx
@@ -8,15 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\mnewsted\local-DA-easyforms-dev\sources\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3C4E1BBD-C5A1-45D0-A20A-113D6283100E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{48733896-28C4-4F26-A176-358AC3A6A676}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-36270" yWindow="-3630" windowWidth="32625" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-35790" yWindow="-2115" windowWidth="32625" windowHeight="15495" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -10038,10 +10037,546 @@
     </r>
   </si>
   <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
+% if get_config("interview page pre"):
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ get_config("interview page pre") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">Haz clic en el nombre de un Formulario Fácil para seguir trabajando en él o para descargar tus formularios completados.
+Usa la acción de etiqueta </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>:tag:</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> para agregar o editar una descripción.
+**Nota: Los Formularios Fácil se eliminan después de 90 días de inactividad.** Si quieres conservarlos por más tiempo, descarga tus formularios o reanuda el Formulario Fácil para restablecer el temporizador de actividad. 
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;nav aria-label="Page navigation"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% if session_page &gt; 0:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Previo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">    </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Próximo</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/a&gt;&lt;/li&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/ul&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>&lt;/nav&gt;</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% else:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">No tienes ningún Formulario Fácil a medias.
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endif
+</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% for interview in interview_list(filename=current_interview_url)[0]:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">* </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${'!@&lt;a class="xyz" href="' + interview_url(i=current_interview_url, session=interview['session']) + '"&gt;!@' +  interview['title'] +  (' (' + interview.get("subtitle",'') + ')' if interview.get('subtitle') else '')  +"!@&lt;/a&gt;!@" }</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  Última visita </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${format_date(interview['modtime'])}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>, actualmente en la página **</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${interview['dict'].get('_internal',{}).get('steps')}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">**
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF008000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">% endfor
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+[**Ver todos tus Formularios Fáciles guardados**](</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF0000FF"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>${url_of('interviews')}</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>)</t>
+    </r>
+  </si>
+  <si>
     <t>Se produjo un error al intentar cargar esta pantalla.
 Puedes probar alguno de estos pasos para recuperar tu trabajo:
 * Haz clic en **Atrás** y vuelve a intentarlo,
-* [:comment-dots: **Cuéntanos qué pasó**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url_es , easy_form_title=ilao_easy_form_title_es, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=action_argument('error_message'), local=False,reset=1) }){target="_blank"}, o
+* [:comment-dots: **Cuéntanos qué pasó**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=showifdef('ilao_easy_form_url_es', 'ilao_easy_form_url') , easy_form_title=showifdef('ilao_easy_form_title_es', 'ilao_easy_form_title'), easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=action_argument('error_message'), local=False,reset=1) }){target="_blank"}, o
 * Visita la [**ILAO Form Library**](https://es.illinoislegalaid.org/form-library) y prueba otro Easy Form.
 ${ collapse_template(al_formatted_error_message) }</t>
   </si>
@@ -10049,545 +10584,9 @@
     <t>Se produjo un error al intentar cargar esta pantalla.
 Puedes intentar uno de estos pasos para recuperar tu trabajo:
 * Haz clic en **Atrás** y vuelve a intentarlo,
-* [:comment-dots: **Cuéntenos qué pasó.**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=ilao_easy_form_url_es , easy_form_title=ilao_easy_form_title_es, easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }){target="_blank"}, o
+* [:comment-dots: **Cuéntenos qué pasó.**](${ interview_url(i="docassemble.ILAO:feedback.yml", easy_form_interview=showifdef('ilao_easy_form_url_es', 'ilao_easy_form_url') ,easy_form_title=showifdef('ilao_easy_form_title_es', 'ilao_easy_form_title'), easy_form_page=current_context().question_id, easy_form_variable=current_context().variable, easy_form_error_message=urllib.parse.quote(str(action_argument('error_message')), safe=''), local=False,reset=1) }){target="_blank"}, o
 * Visita la [**Biblioteca de formularios de ILAO**](https://es.illinoislegalaid.org/form-library) y prueba otro Formulario Fácil.
 ${ collapse_template(al_formatted_error_message) }</t>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True)) &gt; 0:
-% if get_config("interview page pre"):
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ get_config("interview page pre") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">Haz clic en el nombre de un Formulario Fácil para seguir trabajando en él o para descargar tus formularios completados.
-Usa la acción de etiqueta </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>:tag:</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> para agregar o editar una descripción.
-**Nota: Los Formularios Fácil se eliminan después de 90 días de inactividad.** Si quieres conservarlos por más tiempo, descarga tus formularios o reanuda el Formulario Fácil para restablecer el temporizador de actividad. 
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${ session_list_html(filename=None, limit=20, offset=session_page*20, exclude_filenames=al_sessions_to_exclude_from_interview_list, exclude_newly_started_sessions=True, name_label="Título", date_label="Fecha de modificación", details_label="Progreso", actions_label="Acciones", delete_label="Eliminar", rename_label="Renombrar") }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;nav aria-label="Page navigation"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;ul class="pagination justify-content-center"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% if session_page &gt; 0:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=-1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Previo</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-% if len(get_saved_interview_list(filename=None, filename_to_exclude=al_session_store_default_filename, exclude_filenames=al_sessions_to_exclude_from_interview_list, limit=20, offset=session_page*20, exclude_newly_started_sessions=True)) &gt;= 20:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">    </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;li class="page-item"&gt;&lt;a class="page-link" href="${ url_action("update_page_event", page_increment=1) }"&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Próximo</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/a&gt;&lt;/li&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/ul&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>&lt;/nav&gt;</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% else:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">No tienes ningún Formulario Fácil a medias.
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endif
-</t>
-    </r>
-  </si>
-  <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% for interview in interview_list(filename=current_interview_url)[0]:
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">* </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${'!@&lt;a class="xyz" href="' + interview_url(i=current_interview_url, session=interview['session']) + '"&gt;!@' +  interview['title'] +  (' (' + interview.get("subtitle",'') + ')' if interview.get('subtitle') else '')  +"!@&lt;/a&gt;!@" }</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">  Última visita </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${format_date(interview['modtime'])}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>, actualmente en la página **</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${interview['dict'].get('_internal',{}).get('steps')}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">**
-</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF008000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">% endfor
-</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-[**Ver todos tus Formularios Fáciles guardados**](</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FF0000FF"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>${url_of('interviews')}</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color rgb="FF000000"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>)</t>
-    </r>
   </si>
 </sst>
 </file>
@@ -13174,7 +13173,7 @@
         <v>147</v>
       </c>
       <c r="H83" s="2" t="s">
-        <v>528</v>
+        <v>526</v>
       </c>
     </row>
     <row r="84" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">
@@ -13512,7 +13511,7 @@
         <v>364</v>
       </c>
       <c r="H96" s="2" t="s">
-        <v>525</v>
+        <v>527</v>
       </c>
     </row>
     <row r="97" spans="1:8" x14ac:dyDescent="0.3">
@@ -14474,7 +14473,7 @@
         <v>470</v>
       </c>
       <c r="H133" s="2" t="s">
-        <v>526</v>
+        <v>528</v>
       </c>
     </row>
     <row r="134" spans="1:8" x14ac:dyDescent="0.3">
@@ -15196,7 +15195,7 @@
         <v>374</v>
       </c>
       <c r="H161" s="2" t="s">
-        <v>527</v>
+        <v>525</v>
       </c>
     </row>
     <row r="162" spans="1:8" ht="158.4" x14ac:dyDescent="0.3">

</xml_diff>